<commit_message>
provenance: record each series/sheet as a distinct manifest entry
build_run_manifest deduplicated inputs on source_path alone, so a single
Excel/CSV file feeding several series/sheets collapsed to one manifest
entry. Key the dedup on the full linkage tuple (source_path, sample_id,
series_name, sheet_name) so every distinct input is recorded; a per-path
SHA-256 cache hashes each file once. Regenerate the example outputs so the
manifest lists all 13 inputs.
</commit_message>
<xml_diff>
--- a/output/tables/results_timings.xlsx
+++ b/output/tables/results_timings.xlsx
@@ -527,43 +527,43 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>1567.544300000009</v>
+        <v>2901.073599990923</v>
       </c>
       <c r="E2" t="n">
-        <v>0.4941000006510876</v>
+        <v>0.7893999863881618</v>
       </c>
       <c r="F2" t="n">
-        <v>0.6566000010934658</v>
+        <v>1.008100021863356</v>
       </c>
       <c r="G2" t="n">
-        <v>0.06769999890821055</v>
+        <v>0.3046999918296933</v>
       </c>
       <c r="H2" t="n">
-        <v>1.600999996298924</v>
+        <v>3.447600000072271</v>
       </c>
       <c r="I2" t="n">
-        <v>2.828500000759959</v>
+        <v>5.566700012423098</v>
       </c>
       <c r="J2" t="n">
-        <v>0.4941000006510876</v>
+        <v>0.7893999863881618</v>
       </c>
       <c r="K2" t="n">
-        <v>0.2372000017203391</v>
+        <v>0.3475999983493239</v>
       </c>
       <c r="L2" t="n">
-        <v>0.04520000220509246</v>
+        <v>0.06650001159869134</v>
       </c>
       <c r="M2" t="n">
-        <v>1.49760000203969</v>
+        <v>2.620199986267835</v>
       </c>
       <c r="N2" t="n">
-        <v>10.71959999535466</v>
+        <v>17.94869999866933</v>
       </c>
       <c r="O2" t="n">
-        <v>13.54809999611462</v>
+        <v>23.51540001109242</v>
       </c>
       <c r="P2" t="n">
-        <v>1581.092399996123</v>
+        <v>2924.589000002015</v>
       </c>
     </row>
     <row r="3">
@@ -583,43 +583,43 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>1441.708700003801</v>
+        <v>2815.128399990499</v>
       </c>
       <c r="E3" t="n">
-        <v>0.4941000006510876</v>
+        <v>0.7893999863881618</v>
       </c>
       <c r="F3" t="n">
-        <v>0.6566000010934658</v>
+        <v>1.008100021863356</v>
       </c>
       <c r="G3" t="n">
-        <v>0.04030000127386302</v>
+        <v>0.06329998723231256</v>
       </c>
       <c r="H3" t="n">
-        <v>1.439499996195082</v>
+        <v>2.224399999249727</v>
       </c>
       <c r="I3" t="n">
-        <v>4.325599998992402</v>
+        <v>7.885500002885237</v>
       </c>
       <c r="J3" t="n">
-        <v>0.4941000006510876</v>
+        <v>0.7893999863881618</v>
       </c>
       <c r="K3" t="n">
-        <v>0.2372000017203391</v>
+        <v>0.3475999983493239</v>
       </c>
       <c r="L3" t="n">
-        <v>0.03840000135824084</v>
+        <v>0.06329998723231256</v>
       </c>
       <c r="M3" t="n">
-        <v>1.475800003390759</v>
+        <v>2.456800022628158</v>
       </c>
       <c r="N3" t="n">
-        <v>12.25039999553701</v>
+        <v>20.49309998983517</v>
       </c>
       <c r="O3" t="n">
-        <v>16.57599999452941</v>
+        <v>28.37859999272041</v>
       </c>
       <c r="P3" t="n">
-        <v>1458.28469999833</v>
+        <v>2843.506999983219</v>
       </c>
     </row>
     <row r="4">
@@ -639,43 +639,43 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>1561.221400006616</v>
+        <v>2672.110399988014</v>
       </c>
       <c r="E4" t="n">
-        <v>0.4941000006510876</v>
+        <v>0.7893999863881618</v>
       </c>
       <c r="F4" t="n">
-        <v>0.6566000010934658</v>
+        <v>1.008100021863356</v>
       </c>
       <c r="G4" t="n">
-        <v>0.03900000592693686</v>
+        <v>0.0591999851167202</v>
       </c>
       <c r="H4" t="n">
-        <v>1.454400000511669</v>
+        <v>2.207200013799593</v>
       </c>
       <c r="I4" t="n">
-        <v>5.831399997987319</v>
+        <v>10.17250001314096</v>
       </c>
       <c r="J4" t="n">
-        <v>0.4941000006510876</v>
+        <v>0.7893999863881618</v>
       </c>
       <c r="K4" t="n">
-        <v>0.2372000017203391</v>
+        <v>0.3475999983493239</v>
       </c>
       <c r="L4" t="n">
-        <v>0.03709999873535708</v>
+        <v>0.07340000593103468</v>
       </c>
       <c r="M4" t="n">
-        <v>1.707600000372622</v>
+        <v>2.63869998161681</v>
       </c>
       <c r="N4" t="n">
-        <v>14.00209999701474</v>
+        <v>23.22360000107437</v>
       </c>
       <c r="O4" t="n">
-        <v>19.83349999500206</v>
+        <v>33.39610001421534</v>
       </c>
       <c r="P4" t="n">
-        <v>1581.054900001618</v>
+        <v>2705.50650000223</v>
       </c>
     </row>
     <row r="5">
@@ -695,43 +695,43 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>1609.812799993961</v>
+        <v>2748.10329999309</v>
       </c>
       <c r="E5" t="n">
-        <v>0.4941000006510876</v>
+        <v>0.7893999863881618</v>
       </c>
       <c r="F5" t="n">
-        <v>0.6566000010934658</v>
+        <v>1.008100021863356</v>
       </c>
       <c r="G5" t="n">
-        <v>0.03819999983534217</v>
+        <v>0.05569998756982386</v>
       </c>
       <c r="H5" t="n">
-        <v>1.493600000685547</v>
+        <v>2.256300009321421</v>
       </c>
       <c r="I5" t="n">
-        <v>7.37210000079358</v>
+        <v>12.49940000707284</v>
       </c>
       <c r="J5" t="n">
-        <v>0.4941000006510876</v>
+        <v>0.7893999863881618</v>
       </c>
       <c r="K5" t="n">
-        <v>0.2372000017203391</v>
+        <v>0.3475999983493239</v>
       </c>
       <c r="L5" t="n">
-        <v>0.04099999932805076</v>
+        <v>0.06240000948309898</v>
       </c>
       <c r="M5" t="n">
-        <v>1.60199999663746</v>
+        <v>2.3112999915611</v>
       </c>
       <c r="N5" t="n">
-        <v>15.6591999984812</v>
+        <v>25.61939999577589</v>
       </c>
       <c r="O5" t="n">
-        <v>23.03129999927478</v>
+        <v>38.11880000284873</v>
       </c>
       <c r="P5" t="n">
-        <v>1632.844099993235</v>
+        <v>2786.222099995939</v>
       </c>
     </row>
     <row r="6">
@@ -751,43 +751,43 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>1430.161800002679</v>
+        <v>2525.795900000958</v>
       </c>
       <c r="E6" t="n">
-        <v>0.4941000006510876</v>
+        <v>0.7893999863881618</v>
       </c>
       <c r="F6" t="n">
-        <v>0.6566000010934658</v>
+        <v>1.008100021863356</v>
       </c>
       <c r="G6" t="n">
-        <v>0.03840000135824084</v>
+        <v>0.05740000051446259</v>
       </c>
       <c r="H6" t="n">
-        <v>1.512099996034522</v>
+        <v>2.329499984625727</v>
       </c>
       <c r="I6" t="n">
-        <v>8.93029999861028</v>
+        <v>14.8990000016056</v>
       </c>
       <c r="J6" t="n">
-        <v>0.4941000006510876</v>
+        <v>0.7893999863881618</v>
       </c>
       <c r="K6" t="n">
-        <v>0.2372000017203391</v>
+        <v>0.3475999983493239</v>
       </c>
       <c r="L6" t="n">
-        <v>0.04060000355821103</v>
+        <v>0.05740000051446259</v>
       </c>
       <c r="M6" t="n">
-        <v>1.572599998326041</v>
+        <v>2.313300006790087</v>
       </c>
       <c r="N6" t="n">
-        <v>17.28210000146646</v>
+        <v>28.00630001001991</v>
       </c>
       <c r="O6" t="n">
-        <v>26.21240000007674</v>
+        <v>42.90530001162551</v>
       </c>
       <c r="P6" t="n">
-        <v>1456.374200002756</v>
+        <v>2568.701200012583</v>
       </c>
     </row>
     <row r="7">
@@ -807,43 +807,43 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>1608.698200005165</v>
+        <v>2741.206900012912</v>
       </c>
       <c r="E7" t="n">
-        <v>0.4778999937116168</v>
+        <v>0.7562999962829053</v>
       </c>
       <c r="F7" t="n">
-        <v>0.6030000004102476</v>
+        <v>0.967200001468882</v>
       </c>
       <c r="G7" t="n">
-        <v>0.04629999602911994</v>
+        <v>0.08739999611862004</v>
       </c>
       <c r="H7" t="n">
-        <v>1.503699997556396</v>
+        <v>2.317599981324747</v>
       </c>
       <c r="I7" t="n">
-        <v>2.637099998537451</v>
+        <v>4.14259999524802</v>
       </c>
       <c r="J7" t="n">
-        <v>0.4778999937116168</v>
+        <v>0.7562999962829053</v>
       </c>
       <c r="K7" t="n">
-        <v>0.2022999979089946</v>
+        <v>0.3486000059638172</v>
       </c>
       <c r="L7" t="n">
-        <v>0.04540000372799113</v>
+        <v>0.08210001396946609</v>
       </c>
       <c r="M7" t="n">
-        <v>1.450600000680424</v>
+        <v>2.647499990416691</v>
       </c>
       <c r="N7" t="n">
-        <v>10.27529999555554</v>
+        <v>21.39710000483319</v>
       </c>
       <c r="O7" t="n">
-        <v>12.91239999409299</v>
+        <v>25.53970000008121</v>
       </c>
       <c r="P7" t="n">
-        <v>1621.610599999258</v>
+        <v>2766.746600012993</v>
       </c>
     </row>
     <row r="8">
@@ -863,43 +863,43 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>1380.457600003865</v>
+        <v>2530.90539999539</v>
       </c>
       <c r="E8" t="n">
-        <v>0.4778999937116168</v>
+        <v>0.7562999962829053</v>
       </c>
       <c r="F8" t="n">
-        <v>0.6030000004102476</v>
+        <v>0.967200001468882</v>
       </c>
       <c r="G8" t="n">
-        <v>0.03789999755099416</v>
+        <v>0.06199997733347118</v>
       </c>
       <c r="H8" t="n">
-        <v>1.43200000457</v>
+        <v>2.327299996977672</v>
       </c>
       <c r="I8" t="n">
-        <v>4.118699995160569</v>
+        <v>6.561499991221353</v>
       </c>
       <c r="J8" t="n">
-        <v>0.4778999937116168</v>
+        <v>0.7562999962829053</v>
       </c>
       <c r="K8" t="n">
-        <v>0.2022999979089946</v>
+        <v>0.3486000059638172</v>
       </c>
       <c r="L8" t="n">
-        <v>0.03629999991971999</v>
+        <v>0.06329998723231256</v>
       </c>
       <c r="M8" t="n">
-        <v>1.475099998060614</v>
+        <v>2.324100001715124</v>
       </c>
       <c r="N8" t="n">
-        <v>11.79409999895142</v>
+        <v>23.80870000342838</v>
       </c>
       <c r="O8" t="n">
-        <v>15.91279999411199</v>
+        <v>30.37019999464974</v>
       </c>
       <c r="P8" t="n">
-        <v>1396.370399997977</v>
+        <v>2561.27559999004</v>
       </c>
     </row>
     <row r="9">
@@ -919,43 +919,43 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>1412.539900004049</v>
+        <v>2580.54969998193</v>
       </c>
       <c r="E9" t="n">
-        <v>0.4778999937116168</v>
+        <v>0.7562999962829053</v>
       </c>
       <c r="F9" t="n">
-        <v>0.6030000004102476</v>
+        <v>0.967200001468882</v>
       </c>
       <c r="G9" t="n">
-        <v>0.03619999915827066</v>
+        <v>0.0644999963697046</v>
       </c>
       <c r="H9" t="n">
-        <v>1.452299999073148</v>
+        <v>2.440599986584857</v>
       </c>
       <c r="I9" t="n">
-        <v>5.61559999914607</v>
+        <v>9.093500004382804</v>
       </c>
       <c r="J9" t="n">
-        <v>0.4778999937116168</v>
+        <v>0.7562999962829053</v>
       </c>
       <c r="K9" t="n">
-        <v>0.2022999979089946</v>
+        <v>0.3486000059638172</v>
       </c>
       <c r="L9" t="n">
-        <v>0.04089999856660143</v>
+        <v>0.06479999865405262</v>
       </c>
       <c r="M9" t="n">
-        <v>1.556299997901078</v>
+        <v>2.347100002225488</v>
       </c>
       <c r="N9" t="n">
-        <v>13.40619999973569</v>
+        <v>26.24020000803284</v>
       </c>
       <c r="O9" t="n">
-        <v>19.02179999888176</v>
+        <v>35.33370001241565</v>
       </c>
       <c r="P9" t="n">
-        <v>1431.561700002931</v>
+        <v>2615.883399994345</v>
       </c>
     </row>
     <row r="10">
@@ -975,43 +975,43 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>1511.682600001222</v>
+        <v>2624.272599990945</v>
       </c>
       <c r="E10" t="n">
-        <v>0.4778999937116168</v>
+        <v>0.7562999962829053</v>
       </c>
       <c r="F10" t="n">
-        <v>0.6030000004102476</v>
+        <v>0.967200001468882</v>
       </c>
       <c r="G10" t="n">
-        <v>0.03709999873535708</v>
+        <v>0.07070001447573304</v>
       </c>
       <c r="H10" t="n">
-        <v>1.438200000848155</v>
+        <v>2.438999974401668</v>
       </c>
       <c r="I10" t="n">
-        <v>7.098199996107724</v>
+        <v>11.63399999495596</v>
       </c>
       <c r="J10" t="n">
-        <v>0.4778999937116168</v>
+        <v>0.7562999962829053</v>
       </c>
       <c r="K10" t="n">
-        <v>0.2022999979089946</v>
+        <v>0.3486000059638172</v>
       </c>
       <c r="L10" t="n">
-        <v>0.03760000254260376</v>
+        <v>0.06409999332390726</v>
       </c>
       <c r="M10" t="n">
-        <v>1.723800000036135</v>
+        <v>2.320300001883879</v>
       </c>
       <c r="N10" t="n">
-        <v>15.17819999571657</v>
+        <v>28.64520001458004</v>
       </c>
       <c r="O10" t="n">
-        <v>22.27639999182429</v>
+        <v>40.279200009536</v>
       </c>
       <c r="P10" t="n">
-        <v>1533.958999993047</v>
+        <v>2664.551800000481</v>
       </c>
     </row>
     <row r="11">
@@ -1031,43 +1031,43 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>1454.839499994705</v>
+        <v>2501.723800000036</v>
       </c>
       <c r="E11" t="n">
-        <v>0.4778999937116168</v>
+        <v>0.7562999962829053</v>
       </c>
       <c r="F11" t="n">
-        <v>0.6030000004102476</v>
+        <v>0.967200001468882</v>
       </c>
       <c r="G11" t="n">
-        <v>0.03659999492811039</v>
+        <v>0.08540000999346375</v>
       </c>
       <c r="H11" t="n">
-        <v>1.428399998985697</v>
+        <v>2.527500008000061</v>
       </c>
       <c r="I11" t="n">
-        <v>8.569699995859992</v>
+        <v>18.29509998788126</v>
       </c>
       <c r="J11" t="n">
-        <v>0.4778999937116168</v>
+        <v>0.7562999962829053</v>
       </c>
       <c r="K11" t="n">
-        <v>0.2022999979089946</v>
+        <v>0.3486000059638172</v>
       </c>
       <c r="L11" t="n">
-        <v>0.04240000271238387</v>
+        <v>0.06590000702999532</v>
       </c>
       <c r="M11" t="n">
-        <v>1.48829999670852</v>
+        <v>2.382499980740249</v>
       </c>
       <c r="N11" t="n">
-        <v>16.72569999936968</v>
+        <v>31.11239999998361</v>
       </c>
       <c r="O11" t="n">
-        <v>25.29539999522967</v>
+        <v>49.40749998786487</v>
       </c>
       <c r="P11" t="n">
-        <v>1480.134899989935</v>
+        <v>2551.131299987901</v>
       </c>
     </row>
     <row r="12">
@@ -1087,43 +1087,43 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>1658.161899998959</v>
+        <v>2773.55979999993</v>
       </c>
       <c r="E12" t="n">
-        <v>0.4628999959095381</v>
+        <v>0.7747999916318804</v>
       </c>
       <c r="F12" t="n">
-        <v>0.5907000013394281</v>
+        <v>0.9805999870877713</v>
       </c>
       <c r="G12" t="n">
-        <v>0.04439999611349776</v>
+        <v>0.07459998596459627</v>
       </c>
       <c r="H12" t="n">
-        <v>1.457800004573073</v>
+        <v>2.427800005534664</v>
       </c>
       <c r="I12" t="n">
-        <v>2.561299996159505</v>
+        <v>4.269700002623722</v>
       </c>
       <c r="J12" t="n">
-        <v>0.4628999959095381</v>
+        <v>0.7747999916318804</v>
       </c>
       <c r="K12" t="n">
-        <v>0.2080999984173104</v>
+        <v>0.3473999968264252</v>
       </c>
       <c r="L12" t="n">
-        <v>0.0442000018665567</v>
+        <v>0.07899999036453664</v>
       </c>
       <c r="M12" t="n">
-        <v>1.59160000475822</v>
+        <v>2.38099999842234</v>
       </c>
       <c r="N12" t="n">
-        <v>10.3949999975157</v>
+        <v>16.69399999082088</v>
       </c>
       <c r="O12" t="n">
-        <v>12.9562999936752</v>
+        <v>20.96369999344461</v>
       </c>
       <c r="P12" t="n">
-        <v>1671.118199992634</v>
+        <v>2794.523499993375</v>
       </c>
     </row>
     <row r="13">
@@ -1143,43 +1143,43 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>1433.105100004468</v>
+        <v>2439.215500024147</v>
       </c>
       <c r="E13" t="n">
-        <v>0.4628999959095381</v>
+        <v>0.7747999916318804</v>
       </c>
       <c r="F13" t="n">
-        <v>0.5907000013394281</v>
+        <v>0.9805999870877713</v>
       </c>
       <c r="G13" t="n">
-        <v>0.03760000254260376</v>
+        <v>0.06620000931434333</v>
       </c>
       <c r="H13" t="n">
-        <v>1.456699996197131</v>
+        <v>2.339700004085898</v>
       </c>
       <c r="I13" t="n">
-        <v>4.066699999384582</v>
+        <v>6.705100007820874</v>
       </c>
       <c r="J13" t="n">
-        <v>0.4628999959095381</v>
+        <v>0.7747999916318804</v>
       </c>
       <c r="K13" t="n">
-        <v>0.2080999984173104</v>
+        <v>0.3473999968264252</v>
       </c>
       <c r="L13" t="n">
-        <v>0.03909999941242859</v>
+        <v>0.06270001176744699</v>
       </c>
       <c r="M13" t="n">
-        <v>1.449900002626237</v>
+        <v>2.242499991552904</v>
       </c>
       <c r="N13" t="n">
-        <v>11.89490000251681</v>
+        <v>19.01839999482036</v>
       </c>
       <c r="O13" t="n">
-        <v>15.96160000190139</v>
+        <v>25.72350000264123</v>
       </c>
       <c r="P13" t="n">
-        <v>1449.06670000637</v>
+        <v>2464.939000026789</v>
       </c>
     </row>
     <row r="14">
@@ -1199,43 +1199,43 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>1519.864000001689</v>
+        <v>2512.298299989197</v>
       </c>
       <c r="E14" t="n">
-        <v>0.4628999959095381</v>
+        <v>0.7747999916318804</v>
       </c>
       <c r="F14" t="n">
-        <v>0.5907000013394281</v>
+        <v>0.9805999870877713</v>
       </c>
       <c r="G14" t="n">
-        <v>0.0368999972124584</v>
+        <v>0.06379999103955925</v>
       </c>
       <c r="H14" t="n">
-        <v>1.450399999157526</v>
+        <v>2.341999992495403</v>
       </c>
       <c r="I14" t="n">
-        <v>5.562099999224301</v>
+        <v>9.133599989581853</v>
       </c>
       <c r="J14" t="n">
-        <v>0.4628999959095381</v>
+        <v>0.7747999916318804</v>
       </c>
       <c r="K14" t="n">
-        <v>0.2080999984173104</v>
+        <v>0.3473999968264252</v>
       </c>
       <c r="L14" t="n">
-        <v>0.03680000372696668</v>
+        <v>0.06079999729990959</v>
       </c>
       <c r="M14" t="n">
-        <v>6.375500001013279</v>
+        <v>2.324300003238022</v>
       </c>
       <c r="N14" t="n">
-        <v>18.31829999719048</v>
+        <v>21.42069998080842</v>
       </c>
       <c r="O14" t="n">
-        <v>23.88039999641478</v>
+        <v>30.55429997039028</v>
       </c>
       <c r="P14" t="n">
-        <v>1543.744399998104</v>
+        <v>2542.852599959588</v>
       </c>
     </row>
     <row r="15">
@@ -1255,43 +1255,43 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>1585.848700000497</v>
+        <v>2747.335299995029</v>
       </c>
       <c r="E15" t="n">
-        <v>0.4628999959095381</v>
+        <v>0.7747999916318804</v>
       </c>
       <c r="F15" t="n">
-        <v>0.5907000013394281</v>
+        <v>0.9805999870877713</v>
       </c>
       <c r="G15" t="n">
-        <v>0.03580000338843092</v>
+        <v>0.0610999995842576</v>
       </c>
       <c r="H15" t="n">
-        <v>1.446399997803383</v>
+        <v>2.270700002554804</v>
       </c>
       <c r="I15" t="n">
-        <v>7.052000000840053</v>
+        <v>11.48689998080954</v>
       </c>
       <c r="J15" t="n">
-        <v>0.4628999959095381</v>
+        <v>0.7747999916318804</v>
       </c>
       <c r="K15" t="n">
-        <v>0.2080999984173104</v>
+        <v>0.3473999968264252</v>
       </c>
       <c r="L15" t="n">
-        <v>0.04199999966658652</v>
+        <v>0.07089998689480126</v>
       </c>
       <c r="M15" t="n">
-        <v>1.539200005936436</v>
+        <v>2.361199993174523</v>
       </c>
       <c r="N15" t="n">
-        <v>19.91209999687271</v>
+        <v>23.8686999946367</v>
       </c>
       <c r="O15" t="n">
-        <v>26.96409999771276</v>
+        <v>35.35559997544624</v>
       </c>
       <c r="P15" t="n">
-        <v>1612.81279999821</v>
+        <v>2782.690899970476</v>
       </c>
     </row>
     <row r="16">
@@ -1311,43 +1311,43 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>1461.169999995036</v>
+        <v>2572.674399998505</v>
       </c>
       <c r="E16" t="n">
-        <v>0.4628999959095381</v>
+        <v>0.7747999916318804</v>
       </c>
       <c r="F16" t="n">
-        <v>0.5907000013394281</v>
+        <v>0.9805999870877713</v>
       </c>
       <c r="G16" t="n">
-        <v>0.03579999611247331</v>
+        <v>0.0599999912083149</v>
       </c>
       <c r="H16" t="n">
-        <v>1.449700001103338</v>
+        <v>2.303699991898611</v>
       </c>
       <c r="I16" t="n">
-        <v>8.543399999325629</v>
+        <v>13.86859998456202</v>
       </c>
       <c r="J16" t="n">
-        <v>0.4628999959095381</v>
+        <v>0.7747999916318804</v>
       </c>
       <c r="K16" t="n">
-        <v>0.2080999984173104</v>
+        <v>0.3473999968264252</v>
       </c>
       <c r="L16" t="n">
-        <v>0.03609999839682132</v>
+        <v>0.06300001405179501</v>
       </c>
       <c r="M16" t="n">
-        <v>1.416400002199225</v>
+        <v>2.582699991762638</v>
       </c>
       <c r="N16" t="n">
-        <v>21.37260000017704</v>
+        <v>26.52909999596886</v>
       </c>
       <c r="O16" t="n">
-        <v>29.91599999950267</v>
+        <v>40.39769998053089</v>
       </c>
       <c r="P16" t="n">
-        <v>1491.085999994539</v>
+        <v>2613.072099979036</v>
       </c>
     </row>
     <row r="17">
@@ -1367,43 +1367,43 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>1524.964299998828</v>
+        <v>2720.142600010149</v>
       </c>
       <c r="E17" t="n">
-        <v>0.4654000003938563</v>
+        <v>0.8755000017117709</v>
       </c>
       <c r="F17" t="n">
-        <v>0.5785999965155497</v>
+        <v>1.152200013166294</v>
       </c>
       <c r="G17" t="n">
-        <v>0.04470000567380339</v>
+        <v>0.08789999992586672</v>
       </c>
       <c r="H17" t="n">
-        <v>1.466800000343937</v>
+        <v>2.850299992132932</v>
       </c>
       <c r="I17" t="n">
-        <v>2.560799999628216</v>
+        <v>4.981000005500391</v>
       </c>
       <c r="J17" t="n">
-        <v>0.4654000003938563</v>
+        <v>0.8755000017117709</v>
       </c>
       <c r="K17" t="n">
-        <v>0.2089999979943968</v>
+        <v>0.4032999859191477</v>
       </c>
       <c r="L17" t="n">
-        <v>0.04419999459059909</v>
+        <v>0.1028999977279454</v>
       </c>
       <c r="M17" t="n">
-        <v>1.424200003384613</v>
+        <v>2.933700016001239</v>
       </c>
       <c r="N17" t="n">
-        <v>10.24389999656705</v>
+        <v>20.20619998802431</v>
       </c>
       <c r="O17" t="n">
-        <v>12.80469999619527</v>
+        <v>25.1871999935247</v>
       </c>
       <c r="P17" t="n">
-        <v>1537.768999995023</v>
+        <v>2745.329800003674</v>
       </c>
     </row>
     <row r="18">
@@ -1423,43 +1423,43 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>1636.787100003858</v>
+        <v>2555.490099999588</v>
       </c>
       <c r="E18" t="n">
-        <v>0.4654000003938563</v>
+        <v>0.8755000017117709</v>
       </c>
       <c r="F18" t="n">
-        <v>0.5785999965155497</v>
+        <v>1.152200013166294</v>
       </c>
       <c r="G18" t="n">
-        <v>0.03680000372696668</v>
+        <v>0.08110000635497272</v>
       </c>
       <c r="H18" t="n">
-        <v>1.474099997722078</v>
+        <v>2.889700001105666</v>
       </c>
       <c r="I18" t="n">
-        <v>4.083200001332443</v>
+        <v>7.989900012034923</v>
       </c>
       <c r="J18" t="n">
-        <v>0.4654000003938563</v>
+        <v>0.8755000017117709</v>
       </c>
       <c r="K18" t="n">
-        <v>0.2089999979943968</v>
+        <v>0.4032999859191477</v>
       </c>
       <c r="L18" t="n">
-        <v>0.03510000533424318</v>
+        <v>0.07069998537190259</v>
       </c>
       <c r="M18" t="n">
-        <v>1.423299996531568</v>
+        <v>2.785799995763227</v>
       </c>
       <c r="N18" t="n">
-        <v>11.70930000080261</v>
+        <v>23.08529999572784</v>
       </c>
       <c r="O18" t="n">
-        <v>15.79250000213506</v>
+        <v>31.07520000776276</v>
       </c>
       <c r="P18" t="n">
-        <v>1652.579600005993</v>
+        <v>2586.565300007351</v>
       </c>
     </row>
     <row r="19">
@@ -1479,43 +1479,43 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>1565.067900002759</v>
+        <v>2596.035700000357</v>
       </c>
       <c r="E19" t="n">
-        <v>0.4654000003938563</v>
+        <v>0.8755000017117709</v>
       </c>
       <c r="F19" t="n">
-        <v>0.5785999965155497</v>
+        <v>1.152200013166294</v>
       </c>
       <c r="G19" t="n">
-        <v>0.03550000110408291</v>
+        <v>0.07819998427294195</v>
       </c>
       <c r="H19" t="n">
-        <v>1.496099997893907</v>
+        <v>2.737900009378791</v>
       </c>
       <c r="I19" t="n">
-        <v>5.623899996862747</v>
+        <v>10.83730001118965</v>
       </c>
       <c r="J19" t="n">
-        <v>0.4654000003938563</v>
+        <v>0.8755000017117709</v>
       </c>
       <c r="K19" t="n">
-        <v>0.2089999979943968</v>
+        <v>0.4032999859191477</v>
       </c>
       <c r="L19" t="n">
-        <v>0.0354999938281253</v>
+        <v>0.07360000745393336</v>
       </c>
       <c r="M19" t="n">
-        <v>1.401800000166986</v>
+        <v>2.810200006933883</v>
       </c>
       <c r="N19" t="n">
-        <v>13.16149999911431</v>
+        <v>25.99200000986457</v>
       </c>
       <c r="O19" t="n">
-        <v>18.78539999597706</v>
+        <v>36.82930002105422</v>
       </c>
       <c r="P19" t="n">
-        <v>1583.853299998736</v>
+        <v>2632.865000021411</v>
       </c>
     </row>
     <row r="20">
@@ -1535,43 +1535,43 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>1614.825200005725</v>
+        <v>2727.476800006116</v>
       </c>
       <c r="E20" t="n">
-        <v>0.4654000003938563</v>
+        <v>0.8755000017117709</v>
       </c>
       <c r="F20" t="n">
-        <v>0.5785999965155497</v>
+        <v>1.152200013166294</v>
       </c>
       <c r="G20" t="n">
-        <v>0.03629999991971999</v>
+        <v>0.07349997758865356</v>
       </c>
       <c r="H20" t="n">
-        <v>1.431199998478405</v>
+        <v>2.8269000176806</v>
       </c>
       <c r="I20" t="n">
-        <v>7.099800001014955</v>
+        <v>13.76090000849217</v>
       </c>
       <c r="J20" t="n">
-        <v>0.4654000003938563</v>
+        <v>0.8755000017117709</v>
       </c>
       <c r="K20" t="n">
-        <v>0.2089999979943968</v>
+        <v>0.4032999859191477</v>
       </c>
       <c r="L20" t="n">
-        <v>0.03590000414988026</v>
+        <v>0.07340000593103468</v>
       </c>
       <c r="M20" t="n">
-        <v>1.462699998228345</v>
+        <v>2.571499993791804</v>
       </c>
       <c r="N20" t="n">
-        <v>14.6660000027623</v>
+        <v>28.65950000705197</v>
       </c>
       <c r="O20" t="n">
-        <v>21.76580000377726</v>
+        <v>42.42040001554415</v>
       </c>
       <c r="P20" t="n">
-        <v>1636.591000009503</v>
+        <v>2769.89720002166</v>
       </c>
     </row>
     <row r="21">
@@ -1591,43 +1591,43 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>1456.868599998415</v>
+        <v>2914.14349997649</v>
       </c>
       <c r="E21" t="n">
-        <v>0.4654000003938563</v>
+        <v>0.8755000017117709</v>
       </c>
       <c r="F21" t="n">
-        <v>0.5785999965155497</v>
+        <v>1.152200013166294</v>
       </c>
       <c r="G21" t="n">
-        <v>0.03450000076554716</v>
+        <v>0.07249999907799065</v>
       </c>
       <c r="H21" t="n">
-        <v>1.416800005245022</v>
+        <v>2.890399977331981</v>
       </c>
       <c r="I21" t="n">
-        <v>8.558300003642216</v>
+        <v>16.74389999243431</v>
       </c>
       <c r="J21" t="n">
-        <v>0.4654000003938563</v>
+        <v>0.8755000017117709</v>
       </c>
       <c r="K21" t="n">
-        <v>0.2089999979943968</v>
+        <v>0.4032999859191477</v>
       </c>
       <c r="L21" t="n">
-        <v>0.03680000372696668</v>
+        <v>0.0706000137142837</v>
       </c>
       <c r="M21" t="n">
-        <v>1.460800005588681</v>
+        <v>2.569499978562817</v>
       </c>
       <c r="N21" t="n">
-        <v>16.17019999684999</v>
+        <v>31.3175999908708</v>
       </c>
       <c r="O21" t="n">
-        <v>24.7285000004922</v>
+        <v>48.06149998330511</v>
       </c>
       <c r="P21" t="n">
-        <v>1481.597099998908</v>
+        <v>2962.204999959795</v>
       </c>
     </row>
     <row r="22">
@@ -1647,43 +1647,43 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>1649.78390000033</v>
+        <v>3036.870899988571</v>
       </c>
       <c r="E22" t="n">
-        <v>0.4648999965866096</v>
+        <v>0.8521000272594392</v>
       </c>
       <c r="F22" t="n">
-        <v>0.5912999986321665</v>
+        <v>1.175999990664423</v>
       </c>
       <c r="G22" t="n">
-        <v>0.04569999873638153</v>
+        <v>0.08639998850412667</v>
       </c>
       <c r="H22" t="n">
-        <v>1.493199997639749</v>
+        <v>2.867800008971244</v>
       </c>
       <c r="I22" t="n">
-        <v>2.60060000437079</v>
+        <v>4.99600000330247</v>
       </c>
       <c r="J22" t="n">
-        <v>0.4648999965866096</v>
+        <v>0.8521000272594392</v>
       </c>
       <c r="K22" t="n">
-        <v>0.2072999996016733</v>
+        <v>0.385499995900318</v>
       </c>
       <c r="L22" t="n">
-        <v>0.04459999763639644</v>
+        <v>0.07989999721758068</v>
       </c>
       <c r="M22" t="n">
-        <v>1.485799999500159</v>
+        <v>2.568299998529255</v>
       </c>
       <c r="N22" t="n">
-        <v>10.67530000000261</v>
+        <v>19.10239999415353</v>
       </c>
       <c r="O22" t="n">
-        <v>13.2759000043734</v>
+        <v>24.098399997456</v>
       </c>
       <c r="P22" t="n">
-        <v>1663.059800004703</v>
+        <v>3060.969299986027</v>
       </c>
     </row>
     <row r="23">
@@ -1703,43 +1703,43 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>1515.176799999608</v>
+        <v>2922.615599993151</v>
       </c>
       <c r="E23" t="n">
-        <v>0.4648999965866096</v>
+        <v>0.8521000272594392</v>
       </c>
       <c r="F23" t="n">
-        <v>0.5912999986321665</v>
+        <v>1.175999990664423</v>
       </c>
       <c r="G23" t="n">
-        <v>0.03749999450519681</v>
+        <v>0.07830001413822174</v>
       </c>
       <c r="H23" t="n">
-        <v>1.607899997907225</v>
+        <v>2.70839998847805</v>
       </c>
       <c r="I23" t="n">
-        <v>4.256899999745656</v>
+        <v>7.815599994501099</v>
       </c>
       <c r="J23" t="n">
-        <v>0.4648999965866096</v>
+        <v>0.8521000272594392</v>
       </c>
       <c r="K23" t="n">
-        <v>0.2072999996016733</v>
+        <v>0.385499995900318</v>
       </c>
       <c r="L23" t="n">
-        <v>0.03640000068116933</v>
+        <v>0.06849999772384763</v>
       </c>
       <c r="M23" t="n">
-        <v>1.537800002552103</v>
+        <v>2.640000020619482</v>
       </c>
       <c r="N23" t="n">
-        <v>12.25649999832967</v>
+        <v>21.82559997891076</v>
       </c>
       <c r="O23" t="n">
-        <v>16.51339999807533</v>
+        <v>29.64119997341186</v>
       </c>
       <c r="P23" t="n">
-        <v>1531.690199997684</v>
+        <v>2952.256799966563</v>
       </c>
     </row>
     <row r="24">
@@ -1759,43 +1759,43 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>1499.931900005322</v>
+        <v>2802.633500017691</v>
       </c>
       <c r="E24" t="n">
-        <v>0.4648999965866096</v>
+        <v>0.8521000272594392</v>
       </c>
       <c r="F24" t="n">
-        <v>0.5912999986321665</v>
+        <v>1.175999990664423</v>
       </c>
       <c r="G24" t="n">
-        <v>0.03730000025825575</v>
+        <v>0.06910000229254365</v>
       </c>
       <c r="H24" t="n">
-        <v>1.524799998151138</v>
+        <v>2.684199978830293</v>
       </c>
       <c r="I24" t="n">
-        <v>5.828000001201872</v>
+        <v>10.5885999801103</v>
       </c>
       <c r="J24" t="n">
-        <v>0.4648999965866096</v>
+        <v>0.8521000272594392</v>
       </c>
       <c r="K24" t="n">
-        <v>0.2072999996016733</v>
+        <v>0.385499995900318</v>
       </c>
       <c r="L24" t="n">
-        <v>0.03649999416666105</v>
+        <v>0.0653000024612993</v>
       </c>
       <c r="M24" t="n">
-        <v>1.479800004744902</v>
+        <v>2.866299997549504</v>
       </c>
       <c r="N24" t="n">
-        <v>13.77949999732664</v>
+        <v>24.77170000202022</v>
       </c>
       <c r="O24" t="n">
-        <v>19.60749999852851</v>
+        <v>35.36029998213053</v>
       </c>
       <c r="P24" t="n">
-        <v>1519.53940000385</v>
+        <v>2837.993799999822</v>
       </c>
     </row>
     <row r="25">
@@ -1815,43 +1815,43 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>2095.922599997721</v>
+        <v>3047.877300006803</v>
       </c>
       <c r="E25" t="n">
-        <v>0.4648999965866096</v>
+        <v>0.8521000272594392</v>
       </c>
       <c r="F25" t="n">
-        <v>0.5912999986321665</v>
+        <v>1.175999990664423</v>
       </c>
       <c r="G25" t="n">
-        <v>0.03740000101970509</v>
+        <v>0.06659998325631022</v>
       </c>
       <c r="H25" t="n">
-        <v>1.501100006862544</v>
+        <v>2.798100002110004</v>
       </c>
       <c r="I25" t="n">
-        <v>7.373799999186303</v>
+        <v>13.46799999009818</v>
       </c>
       <c r="J25" t="n">
-        <v>0.4648999965866096</v>
+        <v>0.8521000272594392</v>
       </c>
       <c r="K25" t="n">
-        <v>0.2072999996016733</v>
+        <v>0.385499995900318</v>
       </c>
       <c r="L25" t="n">
-        <v>0.03650000144261867</v>
+        <v>0.06590000702999532</v>
       </c>
       <c r="M25" t="n">
-        <v>1.471900002798066</v>
+        <v>2.919299993664026</v>
       </c>
       <c r="N25" t="n">
-        <v>15.29490000393707</v>
+        <v>27.77169999899343</v>
       </c>
       <c r="O25" t="n">
-        <v>22.66870000312338</v>
+        <v>41.2396999890916</v>
       </c>
       <c r="P25" t="n">
-        <v>2118.591300000844</v>
+        <v>3089.116999995895</v>
       </c>
     </row>
     <row r="26">
@@ -1871,43 +1871,43 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>2087.564399997063</v>
+        <v>2942.029199999524</v>
       </c>
       <c r="E26" t="n">
-        <v>0.4648999965866096</v>
+        <v>0.8521000272594392</v>
       </c>
       <c r="F26" t="n">
-        <v>0.5912999986321665</v>
+        <v>1.175999990664423</v>
       </c>
       <c r="G26" t="n">
-        <v>0.0351999988197349</v>
+        <v>0.06320001557469368</v>
       </c>
       <c r="H26" t="n">
-        <v>1.508900000771973</v>
+        <v>2.508600009605289</v>
       </c>
       <c r="I26" t="n">
-        <v>8.924900001147762</v>
+        <v>16.05379997636192</v>
       </c>
       <c r="J26" t="n">
-        <v>0.4648999965866096</v>
+        <v>0.8521000272594392</v>
       </c>
       <c r="K26" t="n">
-        <v>0.2072999996016733</v>
+        <v>0.385499995900318</v>
       </c>
       <c r="L26" t="n">
-        <v>0.03640000068116933</v>
+        <v>0.06540000322274864</v>
       </c>
       <c r="M26" t="n">
-        <v>1.429199997801334</v>
+        <v>2.838200016412884</v>
       </c>
       <c r="N26" t="n">
-        <v>16.76700000098208</v>
+        <v>30.68909997818992</v>
       </c>
       <c r="O26" t="n">
-        <v>25.69190000212984</v>
+        <v>46.74289995455183</v>
       </c>
       <c r="P26" t="n">
-        <v>2113.256299999193</v>
+        <v>2988.772099954076</v>
       </c>
     </row>
     <row r="27">
@@ -1927,43 +1927,43 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>1651.132200000575</v>
+        <v>2910.836399998516</v>
       </c>
       <c r="E27" t="n">
-        <v>187.4648000011803</v>
+        <v>461.3921999989543</v>
       </c>
       <c r="F27" t="n">
         <v>0</v>
       </c>
       <c r="G27" t="n">
-        <v>0.0135000009322539</v>
+        <v>0.0151999993249774</v>
       </c>
       <c r="H27" t="n">
-        <v>0.1837000017985702</v>
+        <v>0.2562999725341797</v>
       </c>
       <c r="I27" t="n">
-        <v>187.6743999964674</v>
+        <v>461.6698999889195</v>
       </c>
       <c r="J27" t="n">
-        <v>187.4648000011803</v>
+        <v>461.3921999989543</v>
       </c>
       <c r="K27" t="n">
         <v>0</v>
       </c>
       <c r="L27" t="n">
-        <v>0.004800000169780105</v>
+        <v>0.006400019628927112</v>
       </c>
       <c r="M27" t="n">
-        <v>0.1063000017893501</v>
+        <v>0.1447999966330826</v>
       </c>
       <c r="N27" t="n">
-        <v>188.2551999951829</v>
+        <v>462.4672000063583</v>
       </c>
       <c r="O27" t="n">
-        <v>375.9295999916503</v>
+        <v>924.1370999952778</v>
       </c>
       <c r="P27" t="n">
-        <v>2027.061799992225</v>
+        <v>3834.973499993794</v>
       </c>
     </row>
     <row r="28">
@@ -1983,43 +1983,43 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>1484.277700001257</v>
+        <v>2802.40159999812</v>
       </c>
       <c r="E28" t="n">
-        <v>187.4648000011803</v>
+        <v>461.3921999989543</v>
       </c>
       <c r="F28" t="n">
         <v>0</v>
       </c>
       <c r="G28" t="n">
-        <v>0.005699999746866524</v>
+        <v>0.010199990356341</v>
       </c>
       <c r="H28" t="n">
-        <v>0.1151999967987649</v>
+        <v>0.1583000121172518</v>
       </c>
       <c r="I28" t="n">
-        <v>187.808299997414</v>
+        <v>461.8563999829348</v>
       </c>
       <c r="J28" t="n">
-        <v>187.4648000011803</v>
+        <v>461.3921999989543</v>
       </c>
       <c r="K28" t="n">
         <v>0</v>
       </c>
       <c r="L28" t="n">
-        <v>0.003100001777056605</v>
+        <v>0.004200002877041698</v>
       </c>
       <c r="M28" t="n">
-        <v>0.09470000077271834</v>
+        <v>0.142100005177781</v>
       </c>
       <c r="N28" t="n">
-        <v>188.356599996041</v>
+        <v>462.6191999996081</v>
       </c>
       <c r="O28" t="n">
-        <v>376.164899993455</v>
+        <v>924.4755999825429</v>
       </c>
       <c r="P28" t="n">
-        <v>1860.442599994713</v>
+        <v>3726.877199980663</v>
       </c>
     </row>
     <row r="29">
@@ -2039,43 +2039,43 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>1386.364699996193</v>
+        <v>2638.016200013226</v>
       </c>
       <c r="E29" t="n">
-        <v>187.4648000011803</v>
+        <v>461.3921999989543</v>
       </c>
       <c r="F29" t="n">
         <v>0</v>
       </c>
       <c r="G29" t="n">
-        <v>0.004200002877041698</v>
+        <v>0.006499991286545992</v>
       </c>
       <c r="H29" t="n">
-        <v>0.09610000415705144</v>
+        <v>0.1346000062767416</v>
       </c>
       <c r="I29" t="n">
-        <v>187.9149000014877</v>
+        <v>462.0067999931052</v>
       </c>
       <c r="J29" t="n">
-        <v>187.4648000011803</v>
+        <v>461.3921999989543</v>
       </c>
       <c r="K29" t="n">
         <v>0</v>
       </c>
       <c r="L29" t="n">
-        <v>0.003300003299955279</v>
+        <v>0.0124999787658453</v>
       </c>
       <c r="M29" t="n">
-        <v>0.09370000043418258</v>
+        <v>0.1416000013705343</v>
       </c>
       <c r="N29" t="n">
-        <v>188.4569999965606</v>
+        <v>462.7782999887131</v>
       </c>
       <c r="O29" t="n">
-        <v>376.3718999980483</v>
+        <v>924.7850999818183</v>
       </c>
       <c r="P29" t="n">
-        <v>1762.736599994241</v>
+        <v>3562.801299995044</v>
       </c>
     </row>
     <row r="30">
@@ -2095,43 +2095,43 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>1472.074599994812</v>
+        <v>2747.368700016523</v>
       </c>
       <c r="E30" t="n">
-        <v>187.4648000011803</v>
+        <v>461.3921999989543</v>
       </c>
       <c r="F30" t="n">
         <v>0</v>
       </c>
       <c r="G30" t="n">
-        <v>0.003500004822853953</v>
+        <v>0.004600005922839046</v>
       </c>
       <c r="H30" t="n">
-        <v>0.09039999713422731</v>
+        <v>0.1398000167682767</v>
       </c>
       <c r="I30" t="n">
-        <v>188.0130999998073</v>
+        <v>462.1578000078443</v>
       </c>
       <c r="J30" t="n">
-        <v>187.4648000011803</v>
+        <v>461.3921999989543</v>
       </c>
       <c r="K30" t="n">
         <v>0</v>
       </c>
       <c r="L30" t="n">
-        <v>0.003000001015607268</v>
+        <v>0.00480000744573772</v>
       </c>
       <c r="M30" t="n">
-        <v>0.1047999976435676</v>
+        <v>0.1399999891873449</v>
       </c>
       <c r="N30" t="n">
-        <v>188.5691999996197</v>
+        <v>462.9308999865316</v>
       </c>
       <c r="O30" t="n">
-        <v>376.5822999994271</v>
+        <v>925.0886999943759</v>
       </c>
       <c r="P30" t="n">
-        <v>1848.656899994239</v>
+        <v>3672.457400010899</v>
       </c>
     </row>
     <row r="31">
@@ -2151,43 +2151,43 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>1370.806099999754</v>
+        <v>2527.954400022281</v>
       </c>
       <c r="E31" t="n">
-        <v>187.4648000011803</v>
+        <v>461.3921999989543</v>
       </c>
       <c r="F31" t="n">
         <v>0</v>
       </c>
       <c r="G31" t="n">
-        <v>0.003299996023997664</v>
+        <v>0.004500005161389709</v>
       </c>
       <c r="H31" t="n">
-        <v>0.1192000054288656</v>
+        <v>0.1420000044163316</v>
       </c>
       <c r="I31" t="n">
-        <v>188.1397999968613</v>
+        <v>462.310000002617</v>
       </c>
       <c r="J31" t="n">
-        <v>187.4648000011803</v>
+        <v>461.3921999989543</v>
       </c>
       <c r="K31" t="n">
         <v>0</v>
       </c>
       <c r="L31" t="n">
-        <v>0.003200002538505942</v>
+        <v>0.004200002877041698</v>
       </c>
       <c r="M31" t="n">
-        <v>0.09809999755816534</v>
+        <v>0.1359999878332019</v>
       </c>
       <c r="N31" t="n">
-        <v>188.6744000003091</v>
+        <v>463.0763999884948</v>
       </c>
       <c r="O31" t="n">
-        <v>376.8141999971704</v>
+        <v>925.3863999911118</v>
       </c>
       <c r="P31" t="n">
-        <v>1747.620299996925</v>
+        <v>3453.340800013393</v>
       </c>
     </row>
     <row r="32">
@@ -2207,43 +2207,43 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>1432.131099994876</v>
+        <v>2565.103000000818</v>
       </c>
       <c r="E32" t="n">
-        <v>36.9462000016938</v>
+        <v>43.23790001217276</v>
       </c>
       <c r="F32" t="n">
         <v>0</v>
       </c>
       <c r="G32" t="n">
-        <v>0.01119999797083437</v>
+        <v>0.01610000617802143</v>
       </c>
       <c r="H32" t="n">
-        <v>0.1574999987496994</v>
+        <v>0.2456000074744225</v>
       </c>
       <c r="I32" t="n">
-        <v>37.1171000006143</v>
+        <v>43.50320002413355</v>
       </c>
       <c r="J32" t="n">
-        <v>36.9462000016938</v>
+        <v>43.23790001217276</v>
       </c>
       <c r="K32" t="n">
         <v>0</v>
       </c>
       <c r="L32" t="n">
-        <v>0.004399997123982757</v>
+        <v>0.007299997378140688</v>
       </c>
       <c r="M32" t="n">
-        <v>0.1104999973904341</v>
+        <v>0.1472000149078667</v>
       </c>
       <c r="N32" t="n">
-        <v>37.67369999695802</v>
+        <v>44.40130002330989</v>
       </c>
       <c r="O32" t="n">
-        <v>74.79079999757232</v>
+        <v>87.90450004744343</v>
       </c>
       <c r="P32" t="n">
-        <v>1506.921899992449</v>
+        <v>2653.007500048261</v>
       </c>
     </row>
     <row r="33">
@@ -2263,43 +2263,43 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>1422.285300002841</v>
+        <v>2487.607299990486</v>
       </c>
       <c r="E33" t="n">
-        <v>36.9462000016938</v>
+        <v>43.23790001217276</v>
       </c>
       <c r="F33" t="n">
         <v>0</v>
       </c>
       <c r="G33" t="n">
-        <v>0.005000001692678779</v>
+        <v>0.008400005754083395</v>
       </c>
       <c r="H33" t="n">
-        <v>0.105200000689365</v>
+        <v>0.1880999770946801</v>
       </c>
       <c r="I33" t="n">
-        <v>37.23870000249008</v>
+        <v>43.71810000156984</v>
       </c>
       <c r="J33" t="n">
-        <v>36.9462000016938</v>
+        <v>43.23790001217276</v>
       </c>
       <c r="K33" t="n">
         <v>0</v>
       </c>
       <c r="L33" t="n">
-        <v>0.003299996023997664</v>
+        <v>0.004700006684288383</v>
       </c>
       <c r="M33" t="n">
-        <v>0.1000000047497451</v>
+        <v>0.1648000034037977</v>
       </c>
       <c r="N33" t="n">
-        <v>37.78060000331607</v>
+        <v>44.57680002087727</v>
       </c>
       <c r="O33" t="n">
-        <v>75.01930000580614</v>
+        <v>88.29490002244711</v>
       </c>
       <c r="P33" t="n">
-        <v>1497.304600008647</v>
+        <v>2575.902200012933</v>
       </c>
     </row>
     <row r="34">
@@ -2319,43 +2319,43 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>1379.047200003697</v>
+        <v>2360.366400011117</v>
       </c>
       <c r="E34" t="n">
-        <v>36.9462000016938</v>
+        <v>43.23790001217276</v>
       </c>
       <c r="F34" t="n">
         <v>0</v>
       </c>
       <c r="G34" t="n">
-        <v>0.003699999069795012</v>
+        <v>0.006799993570894003</v>
       </c>
       <c r="H34" t="n">
-        <v>0.09590000263415277</v>
+        <v>0.1608000020496547</v>
       </c>
       <c r="I34" t="n">
-        <v>37.34380000241799</v>
+        <v>43.89590001665056</v>
       </c>
       <c r="J34" t="n">
-        <v>36.9462000016938</v>
+        <v>43.23790001217276</v>
       </c>
       <c r="K34" t="n">
         <v>0</v>
       </c>
       <c r="L34" t="n">
-        <v>0.002900000254157931</v>
+        <v>0.005300011252984405</v>
       </c>
       <c r="M34" t="n">
-        <v>0.1699999993434176</v>
+        <v>0.158199982251972</v>
       </c>
       <c r="N34" t="n">
-        <v>37.95689999969909</v>
+        <v>44.74710000795312</v>
       </c>
       <c r="O34" t="n">
-        <v>75.30070000211708</v>
+        <v>88.64300002460368</v>
       </c>
       <c r="P34" t="n">
-        <v>1454.347900005814</v>
+        <v>2449.00940003572</v>
       </c>
     </row>
     <row r="35">
@@ -2375,43 +2375,43 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>1402.883299997484</v>
+        <v>2383.241200004704</v>
       </c>
       <c r="E35" t="n">
-        <v>36.9462000016938</v>
+        <v>43.23790001217276</v>
       </c>
       <c r="F35" t="n">
         <v>0</v>
       </c>
       <c r="G35" t="n">
-        <v>0.003599998308345675</v>
+        <v>0.005700014298781753</v>
       </c>
       <c r="H35" t="n">
-        <v>0.1040999995893799</v>
+        <v>0.1539999793749303</v>
       </c>
       <c r="I35" t="n">
-        <v>37.45619999972405</v>
+        <v>44.06250000465661</v>
       </c>
       <c r="J35" t="n">
-        <v>36.9462000016938</v>
+        <v>43.23790001217276</v>
       </c>
       <c r="K35" t="n">
         <v>0</v>
       </c>
       <c r="L35" t="n">
-        <v>0.005500005499925464</v>
+        <v>0.004799978341907263</v>
       </c>
       <c r="M35" t="n">
-        <v>0.1021999996737577</v>
+        <v>0.1447000249754637</v>
       </c>
       <c r="N35" t="n">
-        <v>38.07010000309674</v>
+        <v>44.90210002404638</v>
       </c>
       <c r="O35" t="n">
-        <v>75.52630000282079</v>
+        <v>88.96460002870299</v>
       </c>
       <c r="P35" t="n">
-        <v>1478.409600000305</v>
+        <v>2472.205800033407</v>
       </c>
     </row>
     <row r="36">
@@ -2431,43 +2431,43 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>1461.164400003327</v>
+        <v>2370.934999984456</v>
       </c>
       <c r="E36" t="n">
-        <v>36.9462000016938</v>
+        <v>43.23790001217276</v>
       </c>
       <c r="F36" t="n">
         <v>0</v>
       </c>
       <c r="G36" t="n">
-        <v>0.00360000558430329</v>
+        <v>0.005299982149153948</v>
       </c>
       <c r="H36" t="n">
-        <v>0.09170000703306869</v>
+        <v>0.1665000163484365</v>
       </c>
       <c r="I36" t="n">
-        <v>37.5551999968593</v>
+        <v>44.24020001897588</v>
       </c>
       <c r="J36" t="n">
-        <v>36.9462000016938</v>
+        <v>43.23790001217276</v>
       </c>
       <c r="K36" t="n">
         <v>0</v>
       </c>
       <c r="L36" t="n">
-        <v>0.003500004822853953</v>
+        <v>0.004600005922839046</v>
       </c>
       <c r="M36" t="n">
-        <v>0.09649999992689118</v>
+        <v>0.1577000075485557</v>
       </c>
       <c r="N36" t="n">
-        <v>38.17410000192467</v>
+        <v>45.06980002042837</v>
       </c>
       <c r="O36" t="n">
-        <v>75.72929999878397</v>
+        <v>89.31000003940426</v>
       </c>
       <c r="P36" t="n">
-        <v>1536.893700002111</v>
+        <v>2460.24500002386</v>
       </c>
     </row>
     <row r="37">
@@ -2487,43 +2487,43 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>1401.9868999967</v>
+        <v>2365.147400007118</v>
       </c>
       <c r="E37" t="n">
-        <v>27.79169999848818</v>
+        <v>43.65779997897334</v>
       </c>
       <c r="F37" t="n">
         <v>0</v>
       </c>
       <c r="G37" t="n">
-        <v>0.009800001862458885</v>
+        <v>0.01819999306462705</v>
       </c>
       <c r="H37" t="n">
-        <v>0.1618999958736822</v>
+        <v>0.3114999854005873</v>
       </c>
       <c r="I37" t="n">
-        <v>27.96510000189301</v>
+        <v>43.99189999094233</v>
       </c>
       <c r="J37" t="n">
-        <v>27.79169999848818</v>
+        <v>43.65779997897334</v>
       </c>
       <c r="K37" t="n">
         <v>0</v>
       </c>
       <c r="L37" t="n">
-        <v>0.004399997123982757</v>
+        <v>0.007000024197623134</v>
       </c>
       <c r="M37" t="n">
-        <v>0.1138000006903894</v>
+        <v>0.1491000002715737</v>
       </c>
       <c r="N37" t="n">
-        <v>28.530800002045</v>
+        <v>44.92679997929372</v>
       </c>
       <c r="O37" t="n">
-        <v>56.495900003938</v>
+        <v>88.91869997023605</v>
       </c>
       <c r="P37" t="n">
-        <v>1458.482800000638</v>
+        <v>2454.066099977354</v>
       </c>
     </row>
     <row r="38">
@@ -2543,43 +2543,43 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>1451.692800001183</v>
+        <v>2605.957499996293</v>
       </c>
       <c r="E38" t="n">
-        <v>27.79169999848818</v>
+        <v>43.65779997897334</v>
       </c>
       <c r="F38" t="n">
         <v>0</v>
       </c>
       <c r="G38" t="n">
-        <v>0.005800000508315861</v>
+        <v>0.01359998714178801</v>
       </c>
       <c r="H38" t="n">
-        <v>0.1045000026351772</v>
+        <v>0.2145000034943223</v>
       </c>
       <c r="I38" t="n">
-        <v>28.08750000258442</v>
+        <v>44.24449999351054</v>
       </c>
       <c r="J38" t="n">
-        <v>27.79169999848818</v>
+        <v>43.65779997897334</v>
       </c>
       <c r="K38" t="n">
         <v>0</v>
       </c>
       <c r="L38" t="n">
-        <v>0.003300003299955279</v>
+        <v>0.004900008207187057</v>
       </c>
       <c r="M38" t="n">
-        <v>0.1029999984893948</v>
+        <v>0.1407999952789396</v>
       </c>
       <c r="N38" t="n">
-        <v>28.64080000290414</v>
+        <v>45.07839999860153</v>
       </c>
       <c r="O38" t="n">
-        <v>56.72830000548856</v>
+        <v>89.32289999211207</v>
       </c>
       <c r="P38" t="n">
-        <v>1508.421100006672</v>
+        <v>2695.280399988405</v>
       </c>
     </row>
     <row r="39">
@@ -2599,43 +2599,43 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>1439.7547999979</v>
+        <v>2469.565699982923</v>
       </c>
       <c r="E39" t="n">
-        <v>27.79169999848818</v>
+        <v>43.65779997897334</v>
       </c>
       <c r="F39" t="n">
         <v>0</v>
       </c>
       <c r="G39" t="n">
-        <v>0.003499997546896338</v>
+        <v>0.008400005754083395</v>
       </c>
       <c r="H39" t="n">
-        <v>0.1029000050039031</v>
+        <v>0.1651000056881458</v>
       </c>
       <c r="I39" t="n">
-        <v>28.19889999955194</v>
+        <v>44.42960000596941</v>
       </c>
       <c r="J39" t="n">
-        <v>27.79169999848818</v>
+        <v>43.65779997897334</v>
       </c>
       <c r="K39" t="n">
         <v>0</v>
       </c>
       <c r="L39" t="n">
-        <v>0.003499997546896338</v>
+        <v>0.004300003638491035</v>
       </c>
       <c r="M39" t="n">
-        <v>0.09770000178832561</v>
+        <v>0.1590000174473971</v>
       </c>
       <c r="N39" t="n">
-        <v>28.74680000240915</v>
+        <v>45.24779997882433</v>
       </c>
       <c r="O39" t="n">
-        <v>56.94570000196109</v>
+        <v>89.67739998479374</v>
       </c>
       <c r="P39" t="n">
-        <v>1496.700499999861</v>
+        <v>2559.243099967716</v>
       </c>
     </row>
     <row r="40">
@@ -2655,43 +2655,43 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>1371.484099996451</v>
+        <v>2594.940600014525</v>
       </c>
       <c r="E40" t="n">
-        <v>27.79169999848818</v>
+        <v>43.65779997897334</v>
       </c>
       <c r="F40" t="n">
         <v>0</v>
       </c>
       <c r="G40" t="n">
-        <v>0.003100001777056605</v>
+        <v>0.005799985956400633</v>
       </c>
       <c r="H40" t="n">
-        <v>0.1008000035653822</v>
+        <v>0.153800006955862</v>
       </c>
       <c r="I40" t="n">
-        <v>28.30680000624852</v>
+        <v>44.59679999854416</v>
       </c>
       <c r="J40" t="n">
-        <v>27.79169999848818</v>
+        <v>43.65779997897334</v>
       </c>
       <c r="K40" t="n">
         <v>0</v>
       </c>
       <c r="L40" t="n">
-        <v>0.003000001015607268</v>
+        <v>0.00589998671784997</v>
       </c>
       <c r="M40" t="n">
-        <v>0.09289999434258789</v>
+        <v>0.1564999984111637</v>
       </c>
       <c r="N40" t="n">
-        <v>28.8460000010673</v>
+        <v>45.41699998662807</v>
       </c>
       <c r="O40" t="n">
-        <v>57.15280000731582</v>
+        <v>90.01379998517223</v>
       </c>
       <c r="P40" t="n">
-        <v>1428.636900003767</v>
+        <v>2684.954399999697</v>
       </c>
     </row>
     <row r="41">
@@ -2711,43 +2711,43 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>1426.632800001244</v>
+        <v>2750.403999991249</v>
       </c>
       <c r="E41" t="n">
-        <v>27.79169999848818</v>
+        <v>43.65779997897334</v>
       </c>
       <c r="F41" t="n">
         <v>0</v>
       </c>
       <c r="G41" t="n">
-        <v>0.003100001777056605</v>
+        <v>0.00480000744573772</v>
       </c>
       <c r="H41" t="n">
-        <v>0.09539999882690609</v>
+        <v>0.1570000022184104</v>
       </c>
       <c r="I41" t="n">
-        <v>28.40880000439938</v>
+        <v>44.76469999644905</v>
       </c>
       <c r="J41" t="n">
-        <v>27.79169999848818</v>
+        <v>43.65779997897334</v>
       </c>
       <c r="K41" t="n">
         <v>0</v>
       </c>
       <c r="L41" t="n">
-        <v>0.003399996785447001</v>
+        <v>0.005399982910603285</v>
       </c>
       <c r="M41" t="n">
-        <v>0.1161000036518089</v>
+        <v>0.1376000000163913</v>
       </c>
       <c r="N41" t="n">
-        <v>28.96870000404306</v>
+        <v>45.57029998977669</v>
       </c>
       <c r="O41" t="n">
-        <v>57.37750000844244</v>
+        <v>90.33499998622574</v>
       </c>
       <c r="P41" t="n">
-        <v>1484.010300009686</v>
+        <v>2840.738999977475</v>
       </c>
     </row>
     <row r="42">
@@ -2767,43 +2767,43 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>1437.223200002336</v>
+        <v>2726.877500012051</v>
       </c>
       <c r="E42" t="n">
-        <v>29.13949999492615</v>
+        <v>46.77829999127425</v>
       </c>
       <c r="F42" t="n">
         <v>0</v>
       </c>
       <c r="G42" t="n">
-        <v>0.01309999788645655</v>
+        <v>0.01980000524781644</v>
       </c>
       <c r="H42" t="n">
-        <v>0.1800999962142669</v>
+        <v>0.2593999961391091</v>
       </c>
       <c r="I42" t="n">
-        <v>29.33479999774136</v>
+        <v>47.06049998640083</v>
       </c>
       <c r="J42" t="n">
-        <v>29.13949999492615</v>
+        <v>46.77829999127425</v>
       </c>
       <c r="K42" t="n">
         <v>0</v>
       </c>
       <c r="L42" t="n">
-        <v>0.005000001692678779</v>
+        <v>0.008699978934600949</v>
       </c>
       <c r="M42" t="n">
-        <v>0.1038999980664812</v>
+        <v>0.1799000019673258</v>
       </c>
       <c r="N42" t="n">
-        <v>29.93289999722037</v>
+        <v>48.14599998644553</v>
       </c>
       <c r="O42" t="n">
-        <v>59.26769999496173</v>
+        <v>95.20649997284636</v>
       </c>
       <c r="P42" t="n">
-        <v>1496.490899997298</v>
+        <v>2822.083999984898</v>
       </c>
     </row>
     <row r="43">
@@ -2823,43 +2823,43 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>1599.783899997419</v>
+        <v>2795.954300003359</v>
       </c>
       <c r="E43" t="n">
-        <v>29.13949999492615</v>
+        <v>46.77829999127425</v>
       </c>
       <c r="F43" t="n">
         <v>0</v>
       </c>
       <c r="G43" t="n">
-        <v>0.005999994755256921</v>
+        <v>0.008600007276982069</v>
       </c>
       <c r="H43" t="n">
-        <v>0.1086999982362613</v>
+        <v>0.1842999772634357</v>
       </c>
       <c r="I43" t="n">
-        <v>29.46359999623382</v>
+        <v>47.27379998075776</v>
       </c>
       <c r="J43" t="n">
-        <v>29.13949999492615</v>
+        <v>46.77829999127425</v>
       </c>
       <c r="K43" t="n">
         <v>0</v>
       </c>
       <c r="L43" t="n">
-        <v>0.003500004822853953</v>
+        <v>0.006299989763647318</v>
       </c>
       <c r="M43" t="n">
-        <v>0.1094999970518984</v>
+        <v>0.1899999915622175</v>
       </c>
       <c r="N43" t="n">
-        <v>30.04969999892637</v>
+        <v>48.35179998190142</v>
       </c>
       <c r="O43" t="n">
-        <v>59.5132999951602</v>
+        <v>95.62559996265918</v>
       </c>
       <c r="P43" t="n">
-        <v>1659.297199992579</v>
+        <v>2891.579899966018</v>
       </c>
     </row>
     <row r="44">
@@ -2879,43 +2879,43 @@
         </is>
       </c>
       <c r="D44" t="n">
-        <v>1477.173699997365</v>
+        <v>2961.914299987257</v>
       </c>
       <c r="E44" t="n">
-        <v>29.13949999492615</v>
+        <v>46.77829999127425</v>
       </c>
       <c r="F44" t="n">
         <v>0</v>
       </c>
       <c r="G44" t="n">
-        <v>0.004300003638491035</v>
+        <v>0.006499991286545992</v>
       </c>
       <c r="H44" t="n">
-        <v>0.1021999996737577</v>
+        <v>0.1888000115286559</v>
       </c>
       <c r="I44" t="n">
-        <v>29.57590000005439</v>
+        <v>47.47829999541864</v>
       </c>
       <c r="J44" t="n">
-        <v>29.13949999492615</v>
+        <v>46.77829999127425</v>
       </c>
       <c r="K44" t="n">
         <v>0</v>
       </c>
       <c r="L44" t="n">
-        <v>0.003200002538505942</v>
+        <v>0.006399990525096655</v>
       </c>
       <c r="M44" t="n">
-        <v>0.3369999976712279</v>
+        <v>0.1686000032350421</v>
       </c>
       <c r="N44" t="n">
-        <v>30.39419999549864</v>
+        <v>48.53390000062063</v>
       </c>
       <c r="O44" t="n">
-        <v>59.97009999555303</v>
+        <v>96.01219999603927</v>
       </c>
       <c r="P44" t="n">
-        <v>1537.143799992919</v>
+        <v>3057.926499983296</v>
       </c>
     </row>
     <row r="45">
@@ -2935,43 +2935,43 @@
         </is>
       </c>
       <c r="D45" t="n">
-        <v>1507.402000002912</v>
+        <v>3900.040500011528</v>
       </c>
       <c r="E45" t="n">
-        <v>29.13949999492615</v>
+        <v>46.77829999127425</v>
       </c>
       <c r="F45" t="n">
         <v>0</v>
       </c>
       <c r="G45" t="n">
-        <v>0.004300003638491035</v>
+        <v>0.00689999433234334</v>
       </c>
       <c r="H45" t="n">
-        <v>0.1294999965466559</v>
+        <v>0.2552000223658979</v>
       </c>
       <c r="I45" t="n">
-        <v>29.71409999736352</v>
+        <v>47.75119997793809</v>
       </c>
       <c r="J45" t="n">
-        <v>29.13949999492615</v>
+        <v>46.77829999127425</v>
       </c>
       <c r="K45" t="n">
         <v>0</v>
       </c>
       <c r="L45" t="n">
-        <v>0.01740000152494758</v>
+        <v>0.008200004231184721</v>
       </c>
       <c r="M45" t="n">
-        <v>0.1824999999371357</v>
+        <v>0.1897000183816999</v>
       </c>
       <c r="N45" t="n">
-        <v>30.61180000077002</v>
+        <v>48.73979999683797</v>
       </c>
       <c r="O45" t="n">
-        <v>60.32589999813354</v>
+        <v>96.49099997477606</v>
       </c>
       <c r="P45" t="n">
-        <v>1567.727900001046</v>
+        <v>3996.531499986304</v>
       </c>
     </row>
     <row r="46">
@@ -2991,43 +2991,43 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>1622.091799996269</v>
+        <v>3882.574899995234</v>
       </c>
       <c r="E46" t="n">
-        <v>29.13949999492615</v>
+        <v>46.77829999127425</v>
       </c>
       <c r="F46" t="n">
         <v>0</v>
       </c>
       <c r="G46" t="n">
-        <v>0.003699999069795012</v>
+        <v>0.007299997378140688</v>
       </c>
       <c r="H46" t="n">
-        <v>0.09780000254977494</v>
+        <v>0.1800000027287751</v>
       </c>
       <c r="I46" t="n">
-        <v>29.81970000109868</v>
+        <v>47.94759998912923</v>
       </c>
       <c r="J46" t="n">
-        <v>29.13949999492615</v>
+        <v>46.77829999127425</v>
       </c>
       <c r="K46" t="n">
         <v>0</v>
       </c>
       <c r="L46" t="n">
-        <v>0.005800000508315861</v>
+        <v>0.00589998671784997</v>
       </c>
       <c r="M46" t="n">
-        <v>0.1214000003528781</v>
+        <v>0.1895000168588012</v>
       </c>
       <c r="N46" t="n">
-        <v>30.74699999706354</v>
+        <v>48.94300000160001</v>
       </c>
       <c r="O46" t="n">
-        <v>60.56669999816222</v>
+        <v>96.89059999072924</v>
       </c>
       <c r="P46" t="n">
-        <v>1682.658499994432</v>
+        <v>3979.465499985963</v>
       </c>
     </row>
     <row r="47">
@@ -3047,43 +3047,43 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>1607.940699999745</v>
+        <v>2812.023500009673</v>
       </c>
       <c r="E47" t="n">
-        <v>30.99569999903906</v>
+        <v>47.46470000827685</v>
       </c>
       <c r="F47" t="n">
         <v>0</v>
       </c>
       <c r="G47" t="n">
-        <v>0.01150000025518239</v>
+        <v>0.0534999999217689</v>
       </c>
       <c r="H47" t="n">
-        <v>0.1885000019683503</v>
+        <v>0.2747999969869852</v>
       </c>
       <c r="I47" t="n">
-        <v>31.1982999992324</v>
+        <v>47.79569999664091</v>
       </c>
       <c r="J47" t="n">
-        <v>30.99569999903906</v>
+        <v>47.46470000827685</v>
       </c>
       <c r="K47" t="n">
         <v>0</v>
       </c>
       <c r="L47" t="n">
-        <v>0.004700006684288383</v>
+        <v>0.006600021151825786</v>
       </c>
       <c r="M47" t="n">
-        <v>0.144899997394532</v>
+        <v>0.1532999740447849</v>
       </c>
       <c r="N47" t="n">
-        <v>31.87500000058208</v>
+        <v>48.6310999840498</v>
       </c>
       <c r="O47" t="n">
-        <v>63.07329999981448</v>
+        <v>96.4267999806907</v>
       </c>
       <c r="P47" t="n">
-        <v>1671.013999999559</v>
+        <v>2908.450299990363</v>
       </c>
     </row>
     <row r="48">
@@ -3103,43 +3103,43 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>1367.023899998458</v>
+        <v>2563.624300004449</v>
       </c>
       <c r="E48" t="n">
-        <v>30.99569999903906</v>
+        <v>47.46470000827685</v>
       </c>
       <c r="F48" t="n">
         <v>0</v>
       </c>
       <c r="G48" t="n">
-        <v>0.01310000516241416</v>
+        <v>0.009600014891475439</v>
       </c>
       <c r="H48" t="n">
-        <v>0.1684999951976351</v>
+        <v>0.1644000003580004</v>
       </c>
       <c r="I48" t="n">
-        <v>31.39699999883305</v>
+        <v>47.98860001028515</v>
       </c>
       <c r="J48" t="n">
-        <v>30.99569999903906</v>
+        <v>47.46470000827685</v>
       </c>
       <c r="K48" t="n">
         <v>0</v>
       </c>
       <c r="L48" t="n">
-        <v>0.003799999831244349</v>
+        <v>0.004700006684288383</v>
       </c>
       <c r="M48" t="n">
-        <v>0.1005000012810342</v>
+        <v>0.1721000007819384</v>
       </c>
       <c r="N48" t="n">
-        <v>31.98320000228705</v>
+        <v>48.8138000073377</v>
       </c>
       <c r="O48" t="n">
-        <v>63.3802000011201</v>
+        <v>96.80240001762286</v>
       </c>
       <c r="P48" t="n">
-        <v>1430.404099999578</v>
+        <v>2660.426700022072</v>
       </c>
     </row>
     <row r="49">
@@ -3159,43 +3159,43 @@
         </is>
       </c>
       <c r="D49" t="n">
-        <v>1503.973200000473</v>
+        <v>2694.25329999649</v>
       </c>
       <c r="E49" t="n">
-        <v>30.99569999903906</v>
+        <v>47.46470000827685</v>
       </c>
       <c r="F49" t="n">
         <v>0</v>
       </c>
       <c r="G49" t="n">
-        <v>0.005699999746866524</v>
+        <v>0.005700014298781753</v>
       </c>
       <c r="H49" t="n">
-        <v>0.09889999637380242</v>
+        <v>0.144599995110184</v>
       </c>
       <c r="I49" t="n">
-        <v>31.51169999910053</v>
+        <v>48.14790000091307</v>
       </c>
       <c r="J49" t="n">
-        <v>30.99569999903906</v>
+        <v>47.46470000827685</v>
       </c>
       <c r="K49" t="n">
         <v>0</v>
       </c>
       <c r="L49" t="n">
-        <v>0.003000001015607268</v>
+        <v>0.005300011252984405</v>
       </c>
       <c r="M49" t="n">
-        <v>0.09580000187270343</v>
+        <v>0.1491999719291925</v>
       </c>
       <c r="N49" t="n">
-        <v>32.08540000196081</v>
+        <v>48.97509998409078</v>
       </c>
       <c r="O49" t="n">
-        <v>63.59710000106134</v>
+        <v>97.12299998500384</v>
       </c>
       <c r="P49" t="n">
-        <v>1567.570300001535</v>
+        <v>2791.376299981494</v>
       </c>
     </row>
     <row r="50">
@@ -3215,43 +3215,43 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>1446.499999998196</v>
+        <v>2509.495300007984</v>
       </c>
       <c r="E50" t="n">
-        <v>30.99569999903906</v>
+        <v>47.46470000827685</v>
       </c>
       <c r="F50" t="n">
         <v>0</v>
       </c>
       <c r="G50" t="n">
-        <v>0.004200002877041698</v>
+        <v>0.005200010491535068</v>
       </c>
       <c r="H50" t="n">
-        <v>0.09839999984251335</v>
+        <v>0.1531000016257167</v>
       </c>
       <c r="I50" t="n">
-        <v>31.61890000046697</v>
+        <v>48.31330000888556</v>
       </c>
       <c r="J50" t="n">
-        <v>30.99569999903906</v>
+        <v>47.46470000827685</v>
       </c>
       <c r="K50" t="n">
         <v>0</v>
       </c>
       <c r="L50" t="n">
-        <v>0.003000001015607268</v>
+        <v>0.004900008207187057</v>
       </c>
       <c r="M50" t="n">
-        <v>0.1029999984893948</v>
+        <v>0.1390999823343009</v>
       </c>
       <c r="N50" t="n">
-        <v>32.19459999672836</v>
+        <v>49.12439998588525</v>
       </c>
       <c r="O50" t="n">
-        <v>63.81349999719532</v>
+        <v>97.43769999477081</v>
       </c>
       <c r="P50" t="n">
-        <v>1510.313499995391</v>
+        <v>2606.933000002755</v>
       </c>
     </row>
     <row r="51">
@@ -3271,43 +3271,43 @@
         </is>
       </c>
       <c r="D51" t="n">
-        <v>1482.020100003865</v>
+        <v>2509.231500007445</v>
       </c>
       <c r="E51" t="n">
-        <v>30.99569999903906</v>
+        <v>47.46470000827685</v>
       </c>
       <c r="F51" t="n">
         <v>0</v>
       </c>
       <c r="G51" t="n">
-        <v>0.003699999069795012</v>
+        <v>0.005699985194951296</v>
       </c>
       <c r="H51" t="n">
-        <v>0.09529999806545675</v>
+        <v>0.1392000121995807</v>
       </c>
       <c r="I51" t="n">
-        <v>31.72169999743346</v>
+        <v>48.46540000289679</v>
       </c>
       <c r="J51" t="n">
-        <v>30.99569999903906</v>
+        <v>47.46470000827685</v>
       </c>
       <c r="K51" t="n">
         <v>0</v>
       </c>
       <c r="L51" t="n">
-        <v>0.003200002538505942</v>
+        <v>0.004600005922839046</v>
       </c>
       <c r="M51" t="n">
-        <v>0.09549999958835542</v>
+        <v>0.1481999934185296</v>
       </c>
       <c r="N51" t="n">
-        <v>32.29719999944791</v>
+        <v>49.2828999995254</v>
       </c>
       <c r="O51" t="n">
-        <v>64.01889999688137</v>
+        <v>97.74830000242218</v>
       </c>
       <c r="P51" t="n">
-        <v>1546.039000000746</v>
+        <v>2606.979800009867</v>
       </c>
     </row>
     <row r="52">
@@ -3327,43 +3327,43 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>1452.578199998243</v>
+        <v>2468.183600023622</v>
       </c>
       <c r="E52" t="n">
-        <v>28.56199999951059</v>
+        <v>43.3474000019487</v>
       </c>
       <c r="F52" t="n">
         <v>0</v>
       </c>
       <c r="G52" t="n">
-        <v>0.01210000482387841</v>
+        <v>0.03580001066438854</v>
       </c>
       <c r="H52" t="n">
-        <v>0.1652999999350868</v>
+        <v>0.2317999897059053</v>
       </c>
       <c r="I52" t="n">
-        <v>28.74169999995502</v>
+        <v>43.61839999910444</v>
       </c>
       <c r="J52" t="n">
-        <v>28.56199999951059</v>
+        <v>43.3474000019487</v>
       </c>
       <c r="K52" t="n">
         <v>0</v>
       </c>
       <c r="L52" t="n">
-        <v>0.004699999408330768</v>
+        <v>0.006599992047995329</v>
       </c>
       <c r="M52" t="n">
-        <v>0.09380000119563192</v>
+        <v>0.155999994603917</v>
       </c>
       <c r="N52" t="n">
-        <v>29.32439999858616</v>
+        <v>44.4357999949716</v>
       </c>
       <c r="O52" t="n">
-        <v>58.06609999854118</v>
+        <v>88.05419999407604</v>
       </c>
       <c r="P52" t="n">
-        <v>1510.644299996784</v>
+        <v>2556.237800017698</v>
       </c>
     </row>
     <row r="53">
@@ -3383,43 +3383,43 @@
         </is>
       </c>
       <c r="D53" t="n">
-        <v>1447.432500004652</v>
+        <v>2349.97049998492</v>
       </c>
       <c r="E53" t="n">
-        <v>28.56199999951059</v>
+        <v>43.3474000019487</v>
       </c>
       <c r="F53" t="n">
         <v>0</v>
       </c>
       <c r="G53" t="n">
-        <v>0.006000002031214535</v>
+        <v>0.009099981980398297</v>
       </c>
       <c r="H53" t="n">
-        <v>0.1204000000143424</v>
+        <v>0.1632000203244388</v>
       </c>
       <c r="I53" t="n">
-        <v>28.88089999760268</v>
+        <v>43.80790001596324</v>
       </c>
       <c r="J53" t="n">
-        <v>28.56199999951059</v>
+        <v>43.3474000019487</v>
       </c>
       <c r="K53" t="n">
         <v>0</v>
       </c>
       <c r="L53" t="n">
-        <v>0.003000001015607268</v>
+        <v>0.005599984433501959</v>
       </c>
       <c r="M53" t="n">
-        <v>0.09510000381851569</v>
+        <v>0.1542000100016594</v>
       </c>
       <c r="N53" t="n">
-        <v>29.42579999944428</v>
+        <v>44.60190000827424</v>
       </c>
       <c r="O53" t="n">
-        <v>58.30669999704696</v>
+        <v>88.40980002423748</v>
       </c>
       <c r="P53" t="n">
-        <v>1505.739200001699</v>
+        <v>2438.380300009158</v>
       </c>
     </row>
     <row r="54">
@@ -3439,43 +3439,43 @@
         </is>
       </c>
       <c r="D54" t="n">
-        <v>1715.153599994665</v>
+        <v>2503.654300002381</v>
       </c>
       <c r="E54" t="n">
-        <v>28.56199999951059</v>
+        <v>43.3474000019487</v>
       </c>
       <c r="F54" t="n">
         <v>0</v>
       </c>
       <c r="G54" t="n">
-        <v>0.00410000211559236</v>
+        <v>0.006400019628927112</v>
       </c>
       <c r="H54" t="n">
-        <v>0.09789999603526667</v>
+        <v>0.1515999902039766</v>
       </c>
       <c r="I54" t="n">
-        <v>28.98939999431605</v>
+        <v>43.9743000024464</v>
       </c>
       <c r="J54" t="n">
-        <v>28.56199999951059</v>
+        <v>43.3474000019487</v>
       </c>
       <c r="K54" t="n">
         <v>0</v>
       </c>
       <c r="L54" t="n">
-        <v>0.00309999450109899</v>
+        <v>0.00480000744573772</v>
       </c>
       <c r="M54" t="n">
-        <v>0.09790000331122428</v>
+        <v>0.139600015245378</v>
       </c>
       <c r="N54" t="n">
-        <v>29.52989999903366</v>
+        <v>44.75210001692176</v>
       </c>
       <c r="O54" t="n">
-        <v>58.5192999933497</v>
+        <v>88.72640001936816</v>
       </c>
       <c r="P54" t="n">
-        <v>1773.672899988014</v>
+        <v>2592.380700021749</v>
       </c>
     </row>
     <row r="55">
@@ -3495,43 +3495,43 @@
         </is>
       </c>
       <c r="D55" t="n">
-        <v>1533.832100001746</v>
+        <v>2324.299800005974</v>
       </c>
       <c r="E55" t="n">
-        <v>28.56199999951059</v>
+        <v>43.3474000019487</v>
       </c>
       <c r="F55" t="n">
         <v>0</v>
       </c>
       <c r="G55" t="n">
-        <v>0.003499997546896338</v>
+        <v>0.005199981387704611</v>
       </c>
       <c r="H55" t="n">
-        <v>0.116900002467446</v>
+        <v>0.139600015245378</v>
       </c>
       <c r="I55" t="n">
-        <v>29.11419999873033</v>
+        <v>44.12510001566261</v>
       </c>
       <c r="J55" t="n">
-        <v>28.56199999951059</v>
+        <v>43.3474000019487</v>
       </c>
       <c r="K55" t="n">
         <v>0</v>
       </c>
       <c r="L55" t="n">
-        <v>0.003200002538505942</v>
+        <v>0.005100009730085731</v>
       </c>
       <c r="M55" t="n">
-        <v>0.09219999628840014</v>
+        <v>0.1474999880883843</v>
       </c>
       <c r="N55" t="n">
-        <v>29.62889999616891</v>
+        <v>44.91019999841228</v>
       </c>
       <c r="O55" t="n">
-        <v>58.74309999489924</v>
+        <v>89.03530001407489</v>
       </c>
       <c r="P55" t="n">
-        <v>1592.575199996645</v>
+        <v>2413.335100020049</v>
       </c>
     </row>
     <row r="56">
@@ -3551,43 +3551,43 @@
         </is>
       </c>
       <c r="D56" t="n">
-        <v>1587.654400005704</v>
+        <v>2411.86920000473</v>
       </c>
       <c r="E56" t="n">
-        <v>28.56199999951059</v>
+        <v>43.3474000019487</v>
       </c>
       <c r="F56" t="n">
         <v>0</v>
       </c>
       <c r="G56" t="n">
-        <v>0.003499997546896338</v>
+        <v>0.004600005922839046</v>
       </c>
       <c r="H56" t="n">
-        <v>0.1004000005195849</v>
+        <v>0.1325999910477549</v>
       </c>
       <c r="I56" t="n">
-        <v>29.22209999815095</v>
+        <v>44.26759999478236</v>
       </c>
       <c r="J56" t="n">
-        <v>28.56199999951059</v>
+        <v>43.3474000019487</v>
       </c>
       <c r="K56" t="n">
         <v>0</v>
       </c>
       <c r="L56" t="n">
-        <v>0.002900000254157931</v>
+        <v>0.004700006684288383</v>
       </c>
       <c r="M56" t="n">
-        <v>0.1063000017893501</v>
+        <v>0.1532999740447849</v>
       </c>
       <c r="N56" t="n">
-        <v>29.74129999347497</v>
+        <v>45.07379999267869</v>
       </c>
       <c r="O56" t="n">
-        <v>58.96339999162592</v>
+        <v>89.34139998746105</v>
       </c>
       <c r="P56" t="n">
-        <v>1646.61779999733</v>
+        <v>2501.210599992191</v>
       </c>
     </row>
     <row r="57">
@@ -3607,43 +3607,43 @@
         </is>
       </c>
       <c r="D57" t="n">
-        <v>1535.866599995643</v>
+        <v>2355.619200010551</v>
       </c>
       <c r="E57" t="n">
-        <v>28.8531000041985</v>
+        <v>41.97510000085458</v>
       </c>
       <c r="F57" t="n">
         <v>0</v>
       </c>
       <c r="G57" t="n">
-        <v>0.01100000372389331</v>
+        <v>0.01459999475628138</v>
       </c>
       <c r="H57" t="n">
-        <v>0.1770000017131679</v>
+        <v>0.2152000088244677</v>
       </c>
       <c r="I57" t="n">
-        <v>29.04309999576071</v>
+        <v>42.20809999969788</v>
       </c>
       <c r="J57" t="n">
-        <v>28.8531000041985</v>
+        <v>41.97510000085458</v>
       </c>
       <c r="K57" t="n">
         <v>0</v>
       </c>
       <c r="L57" t="n">
-        <v>0.004600005922839046</v>
+        <v>0.007300026481971145</v>
       </c>
       <c r="M57" t="n">
-        <v>0.1116999992518686</v>
+        <v>0.1573000045027584</v>
       </c>
       <c r="N57" t="n">
-        <v>29.63900000031572</v>
+        <v>43.07479999260977</v>
       </c>
       <c r="O57" t="n">
-        <v>58.68209999607643</v>
+        <v>85.28289999230765</v>
       </c>
       <c r="P57" t="n">
-        <v>1594.548699991719</v>
+        <v>2440.902100002859</v>
       </c>
     </row>
     <row r="58">
@@ -3663,43 +3663,43 @@
         </is>
       </c>
       <c r="D58" t="n">
-        <v>1410.938399996667</v>
+        <v>2320.282900007442</v>
       </c>
       <c r="E58" t="n">
-        <v>28.8531000041985</v>
+        <v>41.97510000085458</v>
       </c>
       <c r="F58" t="n">
         <v>0</v>
       </c>
       <c r="G58" t="n">
-        <v>0.005400004738476127</v>
+        <v>0.008599978173151612</v>
       </c>
       <c r="H58" t="n">
-        <v>0.1031000065268017</v>
+        <v>0.1710999931674451</v>
       </c>
       <c r="I58" t="n">
-        <v>29.16229999391362</v>
+        <v>42.40539998863824</v>
       </c>
       <c r="J58" t="n">
-        <v>28.8531000041985</v>
+        <v>41.97510000085458</v>
       </c>
       <c r="K58" t="n">
         <v>0</v>
       </c>
       <c r="L58" t="n">
-        <v>0.003499997546896338</v>
+        <v>0.005799985956400633</v>
       </c>
       <c r="M58" t="n">
-        <v>0.09890000364976004</v>
+        <v>0.1564999984111637</v>
       </c>
       <c r="N58" t="n">
-        <v>29.74579999863636</v>
+        <v>43.24329999508336</v>
       </c>
       <c r="O58" t="n">
-        <v>58.90809999254998</v>
+        <v>85.6486999837216</v>
       </c>
       <c r="P58" t="n">
-        <v>1469.846499989217</v>
+        <v>2405.931599991163</v>
       </c>
     </row>
     <row r="59">
@@ -3719,43 +3719,43 @@
         </is>
       </c>
       <c r="D59" t="n">
-        <v>1607.219199999236</v>
+        <v>2440.673499979312</v>
       </c>
       <c r="E59" t="n">
-        <v>28.8531000041985</v>
+        <v>41.97510000085458</v>
       </c>
       <c r="F59" t="n">
         <v>0</v>
       </c>
       <c r="G59" t="n">
-        <v>0.003900000592693686</v>
+        <v>0.006699992809444666</v>
       </c>
       <c r="H59" t="n">
-        <v>0.1274999958695844</v>
+        <v>0.1431000127922744</v>
       </c>
       <c r="I59" t="n">
-        <v>29.29919999587582</v>
+        <v>42.56480000913143</v>
       </c>
       <c r="J59" t="n">
-        <v>28.8531000041985</v>
+        <v>41.97510000085458</v>
       </c>
       <c r="K59" t="n">
         <v>0</v>
       </c>
       <c r="L59" t="n">
-        <v>0.003100001777056605</v>
+        <v>0.005499983672052622</v>
       </c>
       <c r="M59" t="n">
-        <v>0.09969999518943951</v>
+        <v>0.159399991389364</v>
       </c>
       <c r="N59" t="n">
-        <v>29.85229999467265</v>
+        <v>43.4151999943424</v>
       </c>
       <c r="O59" t="n">
-        <v>59.15149999054847</v>
+        <v>85.98000000347383</v>
       </c>
       <c r="P59" t="n">
-        <v>1666.370699989784</v>
+        <v>2526.653499982785</v>
       </c>
     </row>
     <row r="60">
@@ -3775,43 +3775,43 @@
         </is>
       </c>
       <c r="D60" t="n">
-        <v>1488.543399995251</v>
+        <v>2455.325899994932</v>
       </c>
       <c r="E60" t="n">
-        <v>28.8531000041985</v>
+        <v>41.97510000085458</v>
       </c>
       <c r="F60" t="n">
         <v>0</v>
       </c>
       <c r="G60" t="n">
-        <v>0.003499997546896338</v>
+        <v>0.005200010491535068</v>
       </c>
       <c r="H60" t="n">
-        <v>0.1027999969664961</v>
+        <v>0.1629999896977097</v>
       </c>
       <c r="I60" t="n">
-        <v>29.40999999555061</v>
+        <v>42.73879999527708</v>
       </c>
       <c r="J60" t="n">
-        <v>28.8531000041985</v>
+        <v>41.97510000085458</v>
       </c>
       <c r="K60" t="n">
         <v>0</v>
       </c>
       <c r="L60" t="n">
-        <v>0.003000001015607268</v>
+        <v>0.005299982149153948</v>
       </c>
       <c r="M60" t="n">
-        <v>0.09480000153416768</v>
+        <v>0.1431000127922744</v>
       </c>
       <c r="N60" t="n">
-        <v>29.95329999976093</v>
+        <v>43.57010000967421</v>
       </c>
       <c r="O60" t="n">
-        <v>59.36329999531154</v>
+        <v>86.30890000495128</v>
       </c>
       <c r="P60" t="n">
-        <v>1547.906699990563</v>
+        <v>2541.634799999883</v>
       </c>
     </row>
     <row r="61">
@@ -3831,43 +3831,43 @@
         </is>
       </c>
       <c r="D61" t="n">
-        <v>1592.324000004737</v>
+        <v>2476.079199986998</v>
       </c>
       <c r="E61" t="n">
-        <v>28.8531000041985</v>
+        <v>41.97510000085458</v>
       </c>
       <c r="F61" t="n">
         <v>0</v>
       </c>
       <c r="G61" t="n">
-        <v>0.00309999450109899</v>
+        <v>0.005299982149153948</v>
       </c>
       <c r="H61" t="n">
-        <v>0.1021999996737577</v>
+        <v>0.1541000092402101</v>
       </c>
       <c r="I61" t="n">
-        <v>29.51879999454832</v>
+        <v>42.90450000553392</v>
       </c>
       <c r="J61" t="n">
-        <v>28.8531000041985</v>
+        <v>41.97510000085458</v>
       </c>
       <c r="K61" t="n">
         <v>0</v>
       </c>
       <c r="L61" t="n">
-        <v>0.003000001015607268</v>
+        <v>0.00480000744573772</v>
       </c>
       <c r="M61" t="n">
-        <v>0.09750000026542693</v>
+        <v>0.1549999869894236</v>
       </c>
       <c r="N61" t="n">
-        <v>30.05699999630451</v>
+        <v>43.73579999082722</v>
       </c>
       <c r="O61" t="n">
-        <v>59.57579999085283</v>
+        <v>86.64029999636114</v>
       </c>
       <c r="P61" t="n">
-        <v>1651.89979999559</v>
+        <v>2562.719499983359</v>
       </c>
     </row>
     <row r="62">
@@ -3887,43 +3887,43 @@
         </is>
       </c>
       <c r="D62" t="n">
-        <v>1520.725200003653</v>
+        <v>2379.28359999205</v>
       </c>
       <c r="E62" t="n">
-        <v>64.05679999443237</v>
+        <v>101.2831999978516</v>
       </c>
       <c r="F62" t="n">
         <v>0</v>
       </c>
       <c r="G62" t="n">
-        <v>0.0118000025395304</v>
+        <v>0.0211999868042767</v>
       </c>
       <c r="H62" t="n">
-        <v>0.1806999935070053</v>
+        <v>0.3149000112898648</v>
       </c>
       <c r="I62" t="n">
-        <v>64.25119999767048</v>
+        <v>101.6227999934927</v>
       </c>
       <c r="J62" t="n">
-        <v>64.05679999443237</v>
+        <v>101.2831999978516</v>
       </c>
       <c r="K62" t="n">
         <v>0</v>
       </c>
       <c r="L62" t="n">
-        <v>0.004600005922839046</v>
+        <v>0.008199975127354264</v>
       </c>
       <c r="M62" t="n">
-        <v>0.1078000059351325</v>
+        <v>0.1725000038277358</v>
       </c>
       <c r="N62" t="n">
-        <v>64.87669999478385</v>
+        <v>102.6020999997854</v>
       </c>
       <c r="O62" t="n">
-        <v>129.1278999924543</v>
+        <v>204.2248999932781</v>
       </c>
       <c r="P62" t="n">
-        <v>1649.853099996108</v>
+        <v>2583.508499985328</v>
       </c>
     </row>
     <row r="63">
@@ -3943,43 +3943,43 @@
         </is>
       </c>
       <c r="D63" t="n">
-        <v>1406.172400005744</v>
+        <v>2227.033499977551</v>
       </c>
       <c r="E63" t="n">
-        <v>64.05679999443237</v>
+        <v>101.2831999978516</v>
       </c>
       <c r="F63" t="n">
         <v>0</v>
       </c>
       <c r="G63" t="n">
-        <v>0.006299997039604932</v>
+        <v>0.01229997724294662</v>
       </c>
       <c r="H63" t="n">
-        <v>0.1139000014518388</v>
+        <v>0.1995000056922436</v>
       </c>
       <c r="I63" t="n">
-        <v>64.3835000009858</v>
+        <v>101.8578000075649</v>
       </c>
       <c r="J63" t="n">
-        <v>64.05679999443237</v>
+        <v>101.2831999978516</v>
       </c>
       <c r="K63" t="n">
         <v>0</v>
       </c>
       <c r="L63" t="n">
-        <v>0.003299996023997664</v>
+        <v>0.005199981387704611</v>
       </c>
       <c r="M63" t="n">
-        <v>0.1125000053434633</v>
+        <v>0.1763000036589801</v>
       </c>
       <c r="N63" t="n">
-        <v>64.99610000173561</v>
+        <v>102.7903000067454</v>
       </c>
       <c r="O63" t="n">
-        <v>129.3796000027214</v>
+        <v>204.6481000143103</v>
       </c>
       <c r="P63" t="n">
-        <v>1535.552000008465</v>
+        <v>2431.681599991862</v>
       </c>
     </row>
     <row r="64">
@@ -3999,43 +3999,43 @@
         </is>
       </c>
       <c r="D64" t="n">
-        <v>1592.075000000477</v>
+        <v>2361.128100019414</v>
       </c>
       <c r="E64" t="n">
-        <v>64.05679999443237</v>
+        <v>101.2831999978516</v>
       </c>
       <c r="F64" t="n">
         <v>0</v>
       </c>
       <c r="G64" t="n">
-        <v>0.003899993316736072</v>
+        <v>0.007099995855242014</v>
       </c>
       <c r="H64" t="n">
-        <v>0.1048000049195252</v>
+        <v>0.1731000083964318</v>
       </c>
       <c r="I64" t="n">
-        <v>64.50200000108453</v>
+        <v>102.0488000067417</v>
       </c>
       <c r="J64" t="n">
-        <v>64.05679999443237</v>
+        <v>101.2831999978516</v>
       </c>
       <c r="K64" t="n">
         <v>0</v>
       </c>
       <c r="L64" t="n">
-        <v>0.003300003299955279</v>
+        <v>0.005399982910603285</v>
       </c>
       <c r="M64" t="n">
-        <v>0.1259000055142678</v>
+        <v>0.1933000166900456</v>
       </c>
       <c r="N64" t="n">
-        <v>65.12890000158222</v>
+        <v>102.9947000206448</v>
       </c>
       <c r="O64" t="n">
-        <v>129.6309000026667</v>
+        <v>205.0435000273865</v>
       </c>
       <c r="P64" t="n">
-        <v>1721.705900003144</v>
+        <v>2566.1716000468</v>
       </c>
     </row>
     <row r="65">
@@ -4055,43 +4055,43 @@
         </is>
       </c>
       <c r="D65" t="n">
-        <v>1433.628699996916</v>
+        <v>2265.248799987603</v>
       </c>
       <c r="E65" t="n">
-        <v>64.05679999443237</v>
+        <v>101.2831999978516</v>
       </c>
       <c r="F65" t="n">
         <v>0</v>
       </c>
       <c r="G65" t="n">
-        <v>0.004200002877041698</v>
+        <v>0.005700014298781753</v>
       </c>
       <c r="H65" t="n">
-        <v>0.09989999671233818</v>
+        <v>0.1673999940976501</v>
       </c>
       <c r="I65" t="n">
-        <v>64.63629999780096</v>
+        <v>102.2295000148006</v>
       </c>
       <c r="J65" t="n">
-        <v>64.05679999443237</v>
+        <v>101.2831999978516</v>
       </c>
       <c r="K65" t="n">
         <v>0</v>
       </c>
       <c r="L65" t="n">
-        <v>0.003799999831244349</v>
+        <v>0.00589998671784997</v>
       </c>
       <c r="M65" t="n">
-        <v>0.1178999955300242</v>
+        <v>0.1697000116109848</v>
       </c>
       <c r="N65" t="n">
-        <v>65.25529999635182</v>
+        <v>103.1771000125445</v>
       </c>
       <c r="O65" t="n">
-        <v>129.8915999941528</v>
+        <v>205.4066000273451</v>
       </c>
       <c r="P65" t="n">
-        <v>1563.520299991069</v>
+        <v>2470.655400014948</v>
       </c>
     </row>
     <row r="66">
@@ -4111,43 +4111,43 @@
         </is>
       </c>
       <c r="D66" t="n">
-        <v>1438.332799996715</v>
+        <v>2245.764099992812</v>
       </c>
       <c r="E66" t="n">
-        <v>64.05679999443237</v>
+        <v>101.2831999978516</v>
       </c>
       <c r="F66" t="n">
         <v>0</v>
       </c>
       <c r="G66" t="n">
-        <v>0.003200002538505942</v>
+        <v>0.005500012775883079</v>
       </c>
       <c r="H66" t="n">
-        <v>0.1170999967143871</v>
+        <v>0.1698000123724341</v>
       </c>
       <c r="I66" t="n">
-        <v>64.7603999968851</v>
+        <v>102.4118000059389</v>
       </c>
       <c r="J66" t="n">
-        <v>64.05679999443237</v>
+        <v>101.2831999978516</v>
       </c>
       <c r="K66" t="n">
         <v>0</v>
       </c>
       <c r="L66" t="n">
-        <v>0.003599998308345675</v>
+        <v>0.005200010491535068</v>
       </c>
       <c r="M66" t="n">
-        <v>0.1049999991664663</v>
+        <v>0.1845000078901649</v>
       </c>
       <c r="N66" t="n">
-        <v>65.36760000017239</v>
+        <v>103.3731999923475</v>
       </c>
       <c r="O66" t="n">
-        <v>130.1279999970575</v>
+        <v>205.7849999982864</v>
       </c>
       <c r="P66" t="n">
-        <v>1568.460799993773</v>
+        <v>2451.549099991098</v>
       </c>
     </row>
   </sheetData>

</xml_diff>